<commit_message>
Add dish filter and sync the latest food spot list.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB9B1CE-A49F-4C3C-B899-F49109405934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51AE47B2-AD35-4434-989D-5E65F7A74ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10300" yWindow="3870" windowWidth="28800" windowHeight="15910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="990" yWindow="3020" windowWidth="28800" windowHeight="15910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="73">
   <si>
     <t>Chin Chin Eating House</t>
   </si>
@@ -169,6 +169,81 @@
   </si>
   <si>
     <t>Sederhana</t>
+  </si>
+  <si>
+    <t>Tom's Palette</t>
+  </si>
+  <si>
+    <t>Dessert</t>
+  </si>
+  <si>
+    <t>Tian Tian Chicken Rice</t>
+  </si>
+  <si>
+    <t>Milli - Sky Dining, Bar and Lounge</t>
+  </si>
+  <si>
+    <t>Elevated Local</t>
+  </si>
+  <si>
+    <t>People's Park Hainan Chicken Rice</t>
+  </si>
+  <si>
+    <t>Imperial Broth Noodles</t>
+  </si>
+  <si>
+    <t>Northeast</t>
+  </si>
+  <si>
+    <t>BKK Bistro Bar Boat Noodles</t>
+  </si>
+  <si>
+    <t>Dish</t>
+  </si>
+  <si>
+    <t>Chicken Rice</t>
+  </si>
+  <si>
+    <t>Soup</t>
+  </si>
+  <si>
+    <t>Noodles</t>
+  </si>
+  <si>
+    <t>BCM, Noodles</t>
+  </si>
+  <si>
+    <t>KKM, Noodles</t>
+  </si>
+  <si>
+    <t>Cafe</t>
+  </si>
+  <si>
+    <t>Seafood</t>
+  </si>
+  <si>
+    <t>Stingray</t>
+  </si>
+  <si>
+    <t>KBBQ</t>
+  </si>
+  <si>
+    <t>Mookata</t>
+  </si>
+  <si>
+    <t>Nasi Padang</t>
+  </si>
+  <si>
+    <t>Ice Cream</t>
+  </si>
+  <si>
+    <t>Thai, Noodles</t>
+  </si>
+  <si>
+    <t>New Ubin Seafood</t>
+  </si>
+  <si>
+    <t>Tze Char</t>
   </si>
 </sst>
 </file>
@@ -489,18 +564,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.90625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="29.7265625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21" style="1" customWidth="1"/>
-    <col min="4" max="5" width="15.1796875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17.453125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="27.6328125" style="1" customWidth="1"/>
+    <col min="2" max="3" width="29.7265625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21" style="1" customWidth="1"/>
+    <col min="5" max="6" width="15.1796875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.453125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="27.6328125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -508,535 +583,777 @@
         <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="1">
         <v>7</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>15</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" s="1">
         <v>4</v>
       </c>
-      <c r="D3" s="1">
+      <c r="E3" s="1">
         <v>14</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="1">
         <v>11</v>
       </c>
-      <c r="D4" s="1">
+      <c r="E4" s="1">
         <v>20</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="G4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="1">
         <v>11</v>
       </c>
-      <c r="D5" s="1">
+      <c r="E5" s="1">
         <v>20</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F5" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" s="1">
         <v>10</v>
       </c>
-      <c r="D6" s="1">
+      <c r="E6" s="1">
         <v>21</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="1">
         <v>10</v>
       </c>
-      <c r="D7" s="1">
+      <c r="E7" s="1">
         <v>14</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="G7" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="1">
         <v>10</v>
       </c>
-      <c r="D8" s="1">
+      <c r="E8" s="1">
         <v>21</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F8" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="1">
         <v>0</v>
       </c>
-      <c r="D9" s="1">
-        <v>24</v>
-      </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="1">
         <v>24</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" s="1">
         <v>0</v>
       </c>
-      <c r="D10" s="1">
-        <v>24</v>
-      </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="1">
         <v>24</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" s="1">
         <v>10</v>
       </c>
-      <c r="D11" s="1">
+      <c r="E11" s="1">
         <v>22</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F11" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" s="1">
         <v>18</v>
       </c>
-      <c r="D12" s="1">
+      <c r="E12" s="1">
         <v>23</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G12" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" s="1">
         <v>12</v>
       </c>
-      <c r="D13" s="1">
+      <c r="E13" s="1">
         <v>22</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="1">
         <v>12</v>
       </c>
-      <c r="D14" s="1">
+      <c r="E14" s="1">
         <v>3</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F14" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="1">
         <v>12</v>
       </c>
-      <c r="D15" s="1">
+      <c r="E15" s="1">
         <v>3</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F15" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="1">
         <v>17</v>
       </c>
-      <c r="D16" s="1">
+      <c r="E16" s="1">
         <v>0</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F16" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" s="1">
         <v>17</v>
       </c>
-      <c r="D17" s="1">
+      <c r="E17" s="1">
         <v>5</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F17" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="1">
         <v>11</v>
       </c>
-      <c r="D18" s="1">
+      <c r="E18" s="1">
         <v>3</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="1">
         <v>0</v>
       </c>
-      <c r="D19" s="1">
-        <v>24</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" s="1">
         <v>24</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="1">
         <v>0</v>
       </c>
-      <c r="D20" s="1">
-        <v>24</v>
-      </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="1">
         <v>24</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D21" s="1">
         <v>12</v>
       </c>
-      <c r="D21" s="1">
+      <c r="E21" s="1">
         <v>5</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F21" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="1">
         <v>11</v>
       </c>
-      <c r="D22" s="1">
+      <c r="E22" s="1">
         <v>4</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F22" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G22" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="1">
         <v>12</v>
       </c>
-      <c r="D23" s="1">
+      <c r="E23" s="1">
         <v>4</v>
       </c>
-      <c r="E23" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G23" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="1">
+      <c r="C24" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D24" s="1">
         <v>12</v>
       </c>
-      <c r="D24" s="1">
+      <c r="E24" s="1">
         <v>6</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F24" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G24" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="1">
         <v>12</v>
       </c>
-      <c r="D25" s="1">
+      <c r="E25" s="1">
         <v>0</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F25" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D26" s="1">
         <v>7</v>
       </c>
-      <c r="D26" s="1">
+      <c r="E26" s="1">
         <v>17</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="F26" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G26" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="1">
+      <c r="C27" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D27" s="1">
         <v>8</v>
       </c>
-      <c r="D27" s="1">
+      <c r="E27" s="1">
         <v>17</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F27" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" s="1">
+        <v>12</v>
+      </c>
+      <c r="E28" s="1">
+        <v>22</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="1">
+        <v>9</v>
+      </c>
+      <c r="E29" s="1">
+        <v>20</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="1">
+        <v>11</v>
+      </c>
+      <c r="E30" s="1">
+        <v>3</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" s="1">
+        <v>0</v>
+      </c>
+      <c r="E31" s="1">
+        <v>24</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D32" s="1">
+        <v>9</v>
+      </c>
+      <c r="E32" s="1">
+        <v>20</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D33" s="1">
+        <v>12</v>
+      </c>
+      <c r="E33" s="1">
+        <v>2</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D34" s="1">
+        <v>11</v>
+      </c>
+      <c r="E34" s="1">
+        <v>1</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync dish tags after removing non-signature dishes.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51AE47B2-AD35-4434-989D-5E65F7A74ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF58976-EE11-4F86-9F9B-A52EFC330A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="990" yWindow="3020" windowWidth="28800" windowHeight="15910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="73">
   <si>
     <t>Chin Chin Eating House</t>
   </si>
@@ -237,13 +237,13 @@
     <t>Ice Cream</t>
   </si>
   <si>
-    <t>Thai, Noodles</t>
-  </si>
-  <si>
     <t>New Ubin Seafood</t>
   </si>
   <si>
     <t>Tze Char</t>
+  </si>
+  <si>
+    <t>Mala</t>
   </si>
 </sst>
 </file>
@@ -881,9 +881,6 @@
       <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="D14" s="1">
         <v>12</v>
       </c>
@@ -904,9 +901,6 @@
       <c r="B15" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="D15" s="1">
         <v>12</v>
       </c>
@@ -927,9 +921,6 @@
       <c r="B16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="D16" s="1">
         <v>17</v>
       </c>
@@ -973,9 +964,6 @@
       <c r="B18" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D18" s="1">
         <v>11</v>
       </c>
@@ -1019,9 +1007,6 @@
       <c r="B20" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="D20" s="1">
         <v>0</v>
       </c>
@@ -1066,7 +1051,7 @@
         <v>39</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="D22" s="1">
         <v>11</v>
@@ -1088,9 +1073,6 @@
       <c r="B23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D23" s="1">
         <v>12</v>
       </c>
@@ -1134,9 +1116,6 @@
       <c r="B25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="D25" s="1">
         <v>12</v>
       </c>
@@ -1249,9 +1228,6 @@
       <c r="B30" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="D30" s="1">
         <v>11</v>
       </c>
@@ -1319,7 +1295,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D33" s="1">
         <v>12</v>
@@ -1336,13 +1312,13 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="D34" s="1">
         <v>11</v>

</xml_diff>

<commit_message>
Add a new food spot to the shared Excel list.
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF58976-EE11-4F86-9F9B-A52EFC330A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD15490B-7B62-4E73-8F46-801A5709D382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="990" yWindow="3020" windowWidth="28800" windowHeight="15910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="75">
   <si>
     <t>Chin Chin Eating House</t>
   </si>
@@ -244,6 +244,12 @@
   </si>
   <si>
     <t>Mala</t>
+  </si>
+  <si>
+    <t>Satori Yakitori</t>
+  </si>
+  <si>
+    <t>Yakitori</t>
   </si>
 </sst>
 </file>
@@ -564,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.90625" style="1" customWidth="1"/>
@@ -1333,6 +1339,29 @@
         <v>19</v>
       </c>
     </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D35" s="1">
+        <v>15</v>
+      </c>
+      <c r="E35" s="1">
+        <v>23</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new food spots to the shared Excel list.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\Projects\food-spot-selector\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\OneDrive\Documents\Cursor Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD15490B-7B62-4E73-8F46-801A5709D382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E6EE4E8-CA3C-4EC3-A541-FBEA2CA206D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="990" yWindow="3020" windowWidth="28800" windowHeight="15910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="12549" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="82">
   <si>
     <t>Chin Chin Eating House</t>
   </si>
@@ -250,6 +250,27 @@
   </si>
   <si>
     <t>Yakitori</t>
+  </si>
+  <si>
+    <t>Ah Boy Chicken Rice</t>
+  </si>
+  <si>
+    <t>Monarchs &amp; Milkweed</t>
+  </si>
+  <si>
+    <t>East</t>
+  </si>
+  <si>
+    <t>Central, East</t>
+  </si>
+  <si>
+    <t>Hi Stranger</t>
+  </si>
+  <si>
+    <t>Bar</t>
+  </si>
+  <si>
+    <t>Sun, Mon</t>
   </si>
 </sst>
 </file>
@@ -570,18 +591,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H38"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.90625" style="1" customWidth="1"/>
-    <col min="2" max="3" width="29.7265625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.921875" style="1" customWidth="1"/>
+    <col min="2" max="3" width="29.69140625" style="1" customWidth="1"/>
     <col min="4" max="4" width="21" style="1" customWidth="1"/>
-    <col min="5" max="6" width="15.1796875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.453125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="27.6328125" style="1" customWidth="1"/>
+    <col min="5" max="6" width="15.15234375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.4609375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="27.61328125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -604,7 +625,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -627,7 +648,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -650,7 +671,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -673,7 +694,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -696,7 +717,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="58.3" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
@@ -719,7 +740,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -742,7 +763,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -765,7 +786,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -788,7 +809,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -811,7 +832,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -834,7 +855,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
@@ -857,7 +878,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
@@ -880,7 +901,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
@@ -900,7 +921,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
@@ -920,7 +941,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
         <v>29</v>
       </c>
@@ -940,7 +961,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
         <v>30</v>
       </c>
@@ -963,7 +984,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
@@ -983,7 +1004,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
         <v>35</v>
       </c>
@@ -1006,7 +1027,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
         <v>36</v>
       </c>
@@ -1026,7 +1047,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
         <v>37</v>
       </c>
@@ -1049,7 +1070,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>38</v>
       </c>
@@ -1072,7 +1093,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
         <v>41</v>
       </c>
@@ -1092,7 +1113,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>42</v>
       </c>
@@ -1115,7 +1136,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
         <v>44</v>
       </c>
@@ -1135,7 +1156,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
         <v>45</v>
       </c>
@@ -1158,7 +1179,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>47</v>
       </c>
@@ -1181,7 +1202,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
         <v>48</v>
       </c>
@@ -1204,7 +1225,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
         <v>50</v>
       </c>
@@ -1224,10 +1245,10 @@
         <v>23</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>51</v>
       </c>
@@ -1247,7 +1268,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="43.75" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>53</v>
       </c>
@@ -1270,7 +1291,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A32" s="1" t="s">
         <v>54</v>
       </c>
@@ -1293,7 +1314,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
         <v>56</v>
       </c>
@@ -1316,7 +1337,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
         <v>70</v>
       </c>
@@ -1339,7 +1360,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
         <v>73</v>
       </c>
@@ -1359,6 +1380,72 @@
         <v>18</v>
       </c>
       <c r="G35" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
+      <c r="A36" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D36" s="1">
+        <v>10</v>
+      </c>
+      <c r="E36" s="1">
+        <v>20</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
+      <c r="A37" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D37" s="1">
+        <v>10</v>
+      </c>
+      <c r="E37" s="1">
+        <v>22</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A38" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D38" s="1">
+        <v>18</v>
+      </c>
+      <c r="E38" s="1">
+        <v>23</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G38" s="1" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add mee hoon kueh spots to the shared Excel list.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\OneDrive\Documents\Cursor Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F72AB2-19EB-4B6B-ABDE-C5A2E6F3F507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5FC7E4-DC8B-4607-BE6A-1BD2EC185A3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="12549" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="251">
   <si>
     <t>Place</t>
   </si>
@@ -232,7 +232,7 @@
     <t>Imperial Broth Noodles</t>
   </si>
   <si>
-    <t>Northeast</t>
+    <t>East</t>
   </si>
   <si>
     <t>BKK Bistro Bar Boat Noodles</t>
@@ -256,9 +256,6 @@
     <t>Monarchs &amp; Milkweed</t>
   </si>
   <si>
-    <t>East</t>
-  </si>
-  <si>
     <t>Hi Stranger</t>
   </si>
   <si>
@@ -373,273 +370,315 @@
     <t>Yi Pin Wei Braised Duck Kway Chap</t>
   </si>
   <si>
+    <t>Braised Duck Rice</t>
+  </si>
+  <si>
+    <t>A Noodle Story</t>
+  </si>
+  <si>
+    <t>Adam Road Noo Cheng Big Prawn Noodle</t>
+  </si>
+  <si>
+    <t>Prawn Noodles, Noodles</t>
+  </si>
+  <si>
+    <t>Alliance Seafood</t>
+  </si>
+  <si>
+    <t>Anglo Indian (Shenton Way)</t>
+  </si>
+  <si>
+    <t>Curry</t>
+  </si>
+  <si>
+    <t>Ar Er Soup</t>
+  </si>
+  <si>
+    <t>Bahrakath Mutton Soup</t>
+  </si>
+  <si>
+    <t>Beach Road Fish Head Bee Hoon</t>
+  </si>
+  <si>
+    <t>Bismillah Biryani (Little India)</t>
+  </si>
+  <si>
+    <t>Biryani</t>
+  </si>
+  <si>
+    <t>Boon Tong Kee (Balestier Road)</t>
+  </si>
+  <si>
+    <t>Chai Chuan Tou Yang Rou Tang</t>
+  </si>
+  <si>
+    <t>Chef Kang's Noodle House</t>
+  </si>
+  <si>
+    <t>Roasted Meats, Noodles</t>
+  </si>
+  <si>
+    <t>Cheok Kee</t>
+  </si>
+  <si>
+    <t>Chey Sua Carrot Cake</t>
+  </si>
+  <si>
+    <t>Carrot Cake</t>
+  </si>
+  <si>
+    <t>Chuan Kee Boneless Braised Duck</t>
+  </si>
+  <si>
+    <t>Cumi Bali</t>
+  </si>
+  <si>
+    <t>Indonesian</t>
+  </si>
+  <si>
+    <t>Da Shi Jia Big Prawn Mee</t>
+  </si>
+  <si>
+    <t>Delhi Lahori</t>
+  </si>
+  <si>
+    <t>Dudu Cooked Food</t>
+  </si>
+  <si>
+    <t>Fei Fei Roasted Noodle</t>
+  </si>
+  <si>
+    <t>Roasted Meats</t>
+  </si>
+  <si>
+    <t>Fico</t>
+  </si>
+  <si>
+    <t>Fu Ming Cooked Food</t>
+  </si>
+  <si>
+    <t>Hai Nan Xing Zhou Beef Noodle</t>
+  </si>
+  <si>
+    <t>Beef Noodles, Noodles</t>
+  </si>
+  <si>
+    <t>Hai Nan Zai</t>
+  </si>
+  <si>
+    <t>Han Kee</t>
+  </si>
+  <si>
+    <t>Heng Heng Cooked Food</t>
+  </si>
+  <si>
+    <t>Heng Kee</t>
+  </si>
+  <si>
+    <t>Curry Chicken Noodles, Noodles</t>
+  </si>
+  <si>
+    <t>Hong Heng Fried Sotong Prawn Mee</t>
+  </si>
+  <si>
+    <t>Hong Kong Yummy Soup</t>
+  </si>
+  <si>
+    <t>Hoo Kee Bak Chang</t>
+  </si>
+  <si>
+    <t>Hui Wei Chilli Ban Mian</t>
+  </si>
+  <si>
+    <t>Chilli Ban Mian, Noodles</t>
+  </si>
+  <si>
+    <t>Indocafé</t>
+  </si>
+  <si>
+    <t>Peranakan</t>
+  </si>
+  <si>
+    <t>J2 Famous Crispy Curry Puff</t>
+  </si>
+  <si>
+    <t>Jalan Sultan Prawn Mee</t>
+  </si>
+  <si>
+    <t>Jason Penang Cuisine</t>
+  </si>
+  <si>
+    <t>Assam Laksa, Noodles</t>
+  </si>
+  <si>
+    <t>Ji De Lai Hainanese Chicken Rice</t>
+  </si>
+  <si>
+    <t>Ji Ji Noodle House</t>
+  </si>
+  <si>
+    <t>Wanton Mee, Noodles</t>
+  </si>
+  <si>
+    <t>Jian Bo Tiong Bahru Shui Kueh</t>
+  </si>
+  <si>
+    <t>Shui Kueh</t>
+  </si>
+  <si>
+    <t>Joo Siah Bak Koot Teh</t>
+  </si>
+  <si>
+    <t>Bak Kut Teh, Soup</t>
+  </si>
+  <si>
+    <t>Jungle Thai</t>
+  </si>
+  <si>
+    <t>Kelantan Kway Chap · Pig Organ Soup</t>
+  </si>
+  <si>
+    <t>Kway Chap, Soup</t>
+  </si>
+  <si>
+    <t>Kitchenman Nasi Lemak</t>
+  </si>
+  <si>
+    <t>Malaysian</t>
+  </si>
+  <si>
+    <t>Nasi Lemak</t>
+  </si>
+  <si>
+    <t>Koh Brother Pig's Organ Soup</t>
+  </si>
+  <si>
+    <t>Kok Sen</t>
+  </si>
+  <si>
+    <t>Kotuwa</t>
+  </si>
+  <si>
+    <t>Sri Lankan</t>
+  </si>
+  <si>
+    <t>Kwang Kee Teochew Fish Porridge</t>
+  </si>
+  <si>
+    <t>Kwee Heng</t>
+  </si>
+  <si>
+    <t>Lagnaa</t>
+  </si>
+  <si>
+    <t>Lai Heng Handmade Teochew Kueh</t>
+  </si>
+  <si>
+    <t>Teochew Kueh, Kueh</t>
+  </si>
+  <si>
+    <t>Lao Fu Zi Fried Kway Teow</t>
+  </si>
+  <si>
+    <t>Fried Kway Teow, Noodles</t>
+  </si>
+  <si>
+    <t>Lian He Ben Ji Claypot</t>
+  </si>
+  <si>
+    <t>Claypot Rice</t>
+  </si>
+  <si>
+    <t>Lixin Teochew Fishball Noodles</t>
+  </si>
+  <si>
+    <t>Fishball Noodles, Noodles</t>
+  </si>
+  <si>
+    <t>North, East, Central, West</t>
+  </si>
+  <si>
+    <t>Margaret Drive Sin Kee Chicken Rice</t>
+  </si>
+  <si>
+    <t>MP Thai (Vision Exchange)</t>
+  </si>
+  <si>
+    <t>Muthu's Curry</t>
+  </si>
+  <si>
+    <t>Na Na Curry</t>
+  </si>
+  <si>
+    <t>Nam Sing Hokkien Fried Mee</t>
+  </si>
+  <si>
+    <t>Hokkien Mee, Noodles</t>
+  </si>
+  <si>
+    <t>New Lucky Claypot Rice</t>
+  </si>
+  <si>
+    <t>No.18 Zion Road Fried Kway Teow</t>
+  </si>
+  <si>
+    <t>Outram Park Fried Kway Teow Mee</t>
+  </si>
+  <si>
+    <t>Ru Ji Kitchen</t>
+  </si>
+  <si>
+    <t>Selamat Datang Warong Pak Sapari</t>
+  </si>
+  <si>
+    <t>Sik Bao Sin</t>
+  </si>
+  <si>
+    <t>Sin Heng Claypot Bak Koot Teh</t>
+  </si>
+  <si>
+    <t>Sin Huat Seafood Restaurant</t>
+  </si>
+  <si>
+    <t>Singapore Fried Hokkien Mee</t>
+  </si>
+  <si>
+    <t>Soh Kee Cooked Food</t>
+  </si>
+  <si>
+    <t>Song Fa Bak Kut Teh (New Bridge Road)</t>
+  </si>
+  <si>
+    <t>Song Fish Soup</t>
+  </si>
+  <si>
+    <t>Song Kee Teochew Fish Porridge</t>
+  </si>
+  <si>
+    <t>Spinach Soup</t>
+  </si>
+  <si>
+    <t>Tai Seng Fish Soup</t>
+  </si>
+  <si>
+    <t>Tai Wah Pork Noodle</t>
+  </si>
+  <si>
+    <t>The Blue Ginger</t>
+  </si>
+  <si>
+    <t>The Coconut Club (Beach Road)</t>
+  </si>
+  <si>
+    <t>Tiong Bahru Hainanese Boneless Chicken Rice</t>
+  </si>
+  <si>
+    <t>To-Ricos Kway Chap</t>
+  </si>
+  <si>
     <t>Kway Chap</t>
   </si>
   <si>
-    <t>A Noodle Story</t>
-  </si>
-  <si>
-    <t>Adam Road Noo Cheng Big Prawn Noodle</t>
-  </si>
-  <si>
-    <t>Alliance Seafood</t>
-  </si>
-  <si>
-    <t>Anglo Indian (Shenton Way)</t>
-  </si>
-  <si>
-    <t>Curry</t>
-  </si>
-  <si>
-    <t>Ar Er Soup</t>
-  </si>
-  <si>
-    <t>Bahrakath Mutton Soup</t>
-  </si>
-  <si>
-    <t>Beach Road Fish Head Bee Hoon</t>
-  </si>
-  <si>
-    <t>Bismillah Biryani (Little India)</t>
-  </si>
-  <si>
-    <t>Biryani</t>
-  </si>
-  <si>
-    <t>Boon Tong Kee (Balestier Road)</t>
-  </si>
-  <si>
-    <t>Chai Chuan Tou Yang Rou Tang</t>
-  </si>
-  <si>
-    <t>Chef Kang's Noodle House</t>
-  </si>
-  <si>
-    <t>Cheok Kee</t>
-  </si>
-  <si>
-    <t>Chey Sua Carrot Cake</t>
-  </si>
-  <si>
-    <t>Carrot Cake</t>
-  </si>
-  <si>
-    <t>Chuan Kee Boneless Braised Duck</t>
-  </si>
-  <si>
-    <t>Cumi Bali</t>
-  </si>
-  <si>
-    <t>Indonesian</t>
-  </si>
-  <si>
-    <t>Da Shi Jia Big Prawn Mee</t>
-  </si>
-  <si>
-    <t>Delhi Lahori</t>
-  </si>
-  <si>
-    <t>Dudu Cooked Food</t>
-  </si>
-  <si>
-    <t>Fei Fei Roasted Noodle</t>
-  </si>
-  <si>
-    <t>Fico</t>
-  </si>
-  <si>
-    <t>Fu Ming Cooked Food</t>
-  </si>
-  <si>
-    <t>Hai Nan Xing Zhou Beef Noodle</t>
-  </si>
-  <si>
-    <t>Hai Nan Zai</t>
-  </si>
-  <si>
-    <t>Han Kee</t>
-  </si>
-  <si>
-    <t>Heng Heng Cooked Food</t>
-  </si>
-  <si>
-    <t>Heng Kee</t>
-  </si>
-  <si>
-    <t>Hong Heng Fried Sotong Prawn Mee</t>
-  </si>
-  <si>
-    <t>Hong Kong Yummy Soup</t>
-  </si>
-  <si>
-    <t>Hoo Kee Bak Chang</t>
-  </si>
-  <si>
-    <t>Hui Wei Chilli Ban Mian</t>
-  </si>
-  <si>
-    <t>Indocafé</t>
-  </si>
-  <si>
-    <t>Peranakan</t>
-  </si>
-  <si>
-    <t>J2 Famous Crispy Curry Puff</t>
-  </si>
-  <si>
-    <t>Jalan Sultan Prawn Mee</t>
-  </si>
-  <si>
-    <t>Jason Penang Cuisine</t>
-  </si>
-  <si>
-    <t>Ji De Lai Hainanese Chicken Rice</t>
-  </si>
-  <si>
-    <t>Ji Ji Noodle House</t>
-  </si>
-  <si>
-    <t>Jian Bo Tiong Bahru Shui Kueh</t>
-  </si>
-  <si>
-    <t>Joo Siah Bak Koot Teh</t>
-  </si>
-  <si>
-    <t>Bak Kut Teh, Soup</t>
-  </si>
-  <si>
-    <t>Jungle Thai</t>
-  </si>
-  <si>
-    <t>Kelantan Kway Chap · Pig Organ Soup</t>
-  </si>
-  <si>
-    <t>Kway Chap, Soup</t>
-  </si>
-  <si>
-    <t>Kitchenman Nasi Lemak</t>
-  </si>
-  <si>
-    <t>Malaysian</t>
-  </si>
-  <si>
-    <t>Nasi Lemak</t>
-  </si>
-  <si>
-    <t>Koh Brother Pig's Organ Soup</t>
-  </si>
-  <si>
-    <t>Kok Sen</t>
-  </si>
-  <si>
-    <t>Kotuwa</t>
-  </si>
-  <si>
-    <t>Sri Lankan</t>
-  </si>
-  <si>
-    <t>Kwang Kee Teochew Fish Porridge</t>
-  </si>
-  <si>
-    <t>Kwee Heng</t>
-  </si>
-  <si>
-    <t>Lagnaa</t>
-  </si>
-  <si>
-    <t>Lai Heng Handmade Teochew Kueh</t>
-  </si>
-  <si>
-    <t>Lao Fu Zi Fried Kway Teow</t>
-  </si>
-  <si>
-    <t>Lian He Ben Ji Claypot</t>
-  </si>
-  <si>
-    <t>Claypot Rice</t>
-  </si>
-  <si>
-    <t>Lixin Teochew Fishball Noodles</t>
-  </si>
-  <si>
-    <t>Margaret Drive Sin Kee Chicken Rice</t>
-  </si>
-  <si>
-    <t>MP Thai (Vision Exchange)</t>
-  </si>
-  <si>
-    <t>Muthu's Curry</t>
-  </si>
-  <si>
-    <t>Na Na Curry</t>
-  </si>
-  <si>
-    <t>Nam Sing Hokkien Fried Mee</t>
-  </si>
-  <si>
-    <t>Hokkien Mee, Noodles</t>
-  </si>
-  <si>
-    <t>New Lucky Claypot Rice</t>
-  </si>
-  <si>
-    <t>No.18 Zion Road Fried Kway Teow</t>
-  </si>
-  <si>
-    <t>Outram Park Fried Kway Teow Mee</t>
-  </si>
-  <si>
-    <t>Ru Ji Kitchen</t>
-  </si>
-  <si>
-    <t>Selamat Datang Warong Pak Sapari</t>
-  </si>
-  <si>
-    <t>Sik Bao Sin</t>
-  </si>
-  <si>
-    <t>Sin Heng Claypot Bak Koot Teh</t>
-  </si>
-  <si>
-    <t>Sin Huat Seafood Restaurant</t>
-  </si>
-  <si>
-    <t>Singapore Fried Hokkien Mee</t>
-  </si>
-  <si>
-    <t>Soh Kee Cooked Food</t>
-  </si>
-  <si>
-    <t>Song Fa Bak Kut Teh (New Bridge Road)</t>
-  </si>
-  <si>
-    <t>Song Fish Soup</t>
-  </si>
-  <si>
-    <t>Song Kee Teochew Fish Porridge</t>
-  </si>
-  <si>
-    <t>Spinach Soup</t>
-  </si>
-  <si>
-    <t>Tai Seng Fish Soup</t>
-  </si>
-  <si>
-    <t>Tai Wah Pork Noodle</t>
-  </si>
-  <si>
-    <t>The Blue Ginger</t>
-  </si>
-  <si>
-    <t>The Coconut Club (Beach Road)</t>
-  </si>
-  <si>
-    <t>Tiong Bahru Hainanese Boneless Chicken Rice</t>
-  </si>
-  <si>
-    <t>To-Ricos Kway Chap</t>
-  </si>
-  <si>
     <t>True Blue Cuisine</t>
   </si>
   <si>
@@ -658,6 +697,9 @@
     <t>Hor Fun, Noodles</t>
   </si>
   <si>
+    <t>Sat, Sun</t>
+  </si>
+  <si>
     <t>Yhingthai Palace</t>
   </si>
   <si>
@@ -673,46 +715,64 @@
     <t>Zhup Zhup Noodles</t>
   </si>
   <si>
-    <t>Braised Duck Rice</t>
-  </si>
-  <si>
-    <t>Roasted Meats</t>
-  </si>
-  <si>
-    <t>Curry Chicken Noodles, Noodles</t>
-  </si>
-  <si>
-    <t>Prawn Noodles, Noodles</t>
-  </si>
-  <si>
-    <t>Roasted Meats, Noodles</t>
-  </si>
-  <si>
-    <t>Beef Noodles, Noodles</t>
-  </si>
-  <si>
-    <t>Chilli Ban Mian, Noodles</t>
-  </si>
-  <si>
-    <t>Assam Laksa, Noodles</t>
-  </si>
-  <si>
-    <t>Wanton Mee, Noodles</t>
-  </si>
-  <si>
-    <t>Shui Kueh</t>
-  </si>
-  <si>
-    <t>Teochew Kueh, Kueh</t>
-  </si>
-  <si>
-    <t>Fried Kway Teow, Noodles</t>
-  </si>
-  <si>
-    <t>Fishball Noodles, Noodles</t>
-  </si>
-  <si>
-    <t>North, East, Central, West</t>
+    <t>Geylang Lor 9 Mee Hoon Kueh</t>
+  </si>
+  <si>
+    <t>Mee Hoon Kueh, Noodles</t>
+  </si>
+  <si>
+    <t>Lor 9 Beef Kway Teow</t>
+  </si>
+  <si>
+    <t>Beef Kway Teow, Noodles</t>
+  </si>
+  <si>
+    <t>Greenview Cafe</t>
+  </si>
+  <si>
+    <t>Madam Tyrant</t>
+  </si>
+  <si>
+    <t>Seletar Sheng Mian &amp; Mian Fen Guo</t>
+  </si>
+  <si>
+    <t>Ah Yi Handmade Noodle</t>
+  </si>
+  <si>
+    <t>Mee Hoon Kueh, Fish Soup, Noodles</t>
+  </si>
+  <si>
+    <t>Ai Chi Mee Hoon Kueh</t>
+  </si>
+  <si>
+    <t>Banting Traditional Cuisine</t>
+  </si>
+  <si>
+    <t>Mee Hoon Kueh, Chilli Ban Mian, Noodles</t>
+  </si>
+  <si>
+    <t>Sat</t>
+  </si>
+  <si>
+    <t>Ge Ge Jia K Kitchen</t>
+  </si>
+  <si>
+    <t>Sky JB Mian Fen Kueh</t>
+  </si>
+  <si>
+    <t>Fri</t>
+  </si>
+  <si>
+    <t>Penang Heng Heng Handmade Noodle</t>
+  </si>
+  <si>
+    <t>Tue</t>
+  </si>
+  <si>
+    <t>Jiak Song Mee Hoon Kway</t>
+  </si>
+  <si>
+    <t>L32 Handmade Noodles</t>
   </si>
 </sst>
 </file>
@@ -1036,7 +1096,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H144"/>
+  <dimension ref="A1:H157"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="16.921875" style="1" customWidth="1"/>
@@ -1871,15 +1931,15 @@
         <v>21</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A38" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="D38" s="1">
         <v>18</v>
@@ -1888,7 +1948,7 @@
         <v>23</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G38" s="1" t="s">
         <v>11</v>
@@ -1896,7 +1956,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A39" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>43</v>
@@ -1916,7 +1976,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>43</v>
@@ -1936,13 +1996,13 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="D41" s="2">
         <v>12</v>
@@ -1954,12 +2014,12 @@
         <v>21</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A42" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>36</v>
@@ -1974,18 +2034,18 @@
         <v>21</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A43" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>58</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D43" s="1">
         <v>9</v>
@@ -2002,13 +2062,13 @@
     </row>
     <row r="44" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A44" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="D44" s="1">
         <v>10</v>
@@ -2025,13 +2085,13 @@
     </row>
     <row r="45" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A45" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D45" s="1">
         <v>10</v>
@@ -2048,7 +2108,7 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A46" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>67</v>
@@ -2068,13 +2128,13 @@
     </row>
     <row r="47" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A47" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D47" s="1">
         <v>11</v>
@@ -2091,7 +2151,7 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A48" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>40</v>
@@ -2114,13 +2174,13 @@
     </row>
     <row r="49" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D49" s="1">
         <v>11</v>
@@ -2137,13 +2197,13 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B50" t="s">
         <v>8</v>
       </c>
       <c r="C50" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D50">
         <v>10</v>
@@ -2155,18 +2215,18 @@
         <v>21</v>
       </c>
       <c r="G50" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
+        <v>99</v>
+      </c>
+      <c r="B51" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" t="s">
         <v>100</v>
-      </c>
-      <c r="B51" t="s">
-        <v>8</v>
-      </c>
-      <c r="C51" t="s">
-        <v>101</v>
       </c>
       <c r="D51">
         <v>17</v>
@@ -2175,7 +2235,7 @@
         <v>0</v>
       </c>
       <c r="F51" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G51" t="s">
         <v>11</v>
@@ -2183,13 +2243,13 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
+        <v>102</v>
+      </c>
+      <c r="B52" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" t="s">
         <v>103</v>
-      </c>
-      <c r="B52" t="s">
-        <v>8</v>
-      </c>
-      <c r="C52" t="s">
-        <v>104</v>
       </c>
       <c r="D52">
         <v>12</v>
@@ -2206,13 +2266,13 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
+        <v>104</v>
+      </c>
+      <c r="B53" t="s">
+        <v>8</v>
+      </c>
+      <c r="C53" t="s">
         <v>105</v>
-      </c>
-      <c r="B53" t="s">
-        <v>8</v>
-      </c>
-      <c r="C53" t="s">
-        <v>106</v>
       </c>
       <c r="D53">
         <v>11</v>
@@ -2224,18 +2284,18 @@
         <v>18</v>
       </c>
       <c r="G53" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
+        <v>106</v>
+      </c>
+      <c r="B54" t="s">
         <v>107</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>108</v>
-      </c>
-      <c r="C54" t="s">
-        <v>109</v>
       </c>
       <c r="D54">
         <v>7</v>
@@ -2244,15 +2304,15 @@
         <v>14</v>
       </c>
       <c r="F54" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G54" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B55" t="s">
         <v>8</v>
@@ -2267,15 +2327,15 @@
         <v>23</v>
       </c>
       <c r="F55" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G55" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B56" t="s">
         <v>8</v>
@@ -2293,17 +2353,16 @@
         <v>10</v>
       </c>
       <c r="G56" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B57" t="s">
         <v>49</v>
       </c>
-      <c r="C57"/>
       <c r="D57">
         <v>11</v>
       </c>
@@ -2319,13 +2378,13 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
+        <v>113</v>
+      </c>
+      <c r="B58" t="s">
+        <v>8</v>
+      </c>
+      <c r="C58" t="s">
         <v>114</v>
-      </c>
-      <c r="B58" t="s">
-        <v>8</v>
-      </c>
-      <c r="C58" t="s">
-        <v>115</v>
       </c>
       <c r="D58">
         <v>5</v>
@@ -2342,13 +2401,13 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
+        <v>115</v>
+      </c>
+      <c r="B59" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" t="s">
         <v>116</v>
-      </c>
-      <c r="B59" t="s">
-        <v>8</v>
-      </c>
-      <c r="C59" t="s">
-        <v>217</v>
       </c>
       <c r="D59">
         <v>6</v>
@@ -2360,12 +2419,12 @@
         <v>21</v>
       </c>
       <c r="G59" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B60" t="s">
         <v>8</v>
@@ -2388,13 +2447,13 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
+        <v>118</v>
+      </c>
+      <c r="B61" t="s">
+        <v>8</v>
+      </c>
+      <c r="C61" t="s">
         <v>119</v>
-      </c>
-      <c r="B61" t="s">
-        <v>8</v>
-      </c>
-      <c r="C61" t="s">
-        <v>220</v>
       </c>
       <c r="D61">
         <v>10</v>
@@ -2437,7 +2496,7 @@
         <v>121</v>
       </c>
       <c r="B63" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C63" t="s">
         <v>122</v>
@@ -2483,7 +2542,7 @@
         <v>124</v>
       </c>
       <c r="B65" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C65" t="s">
         <v>20</v>
@@ -2509,7 +2568,7 @@
         <v>8</v>
       </c>
       <c r="C66" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D66">
         <v>10</v>
@@ -2529,7 +2588,7 @@
         <v>126</v>
       </c>
       <c r="B67" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C67" t="s">
         <v>127</v>
@@ -2601,7 +2660,7 @@
         <v>8</v>
       </c>
       <c r="C70" t="s">
-        <v>221</v>
+        <v>131</v>
       </c>
       <c r="D70">
         <v>11</v>
@@ -2618,13 +2677,13 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B71" t="s">
         <v>8</v>
       </c>
       <c r="C71" t="s">
-        <v>217</v>
+        <v>116</v>
       </c>
       <c r="D71">
         <v>10</v>
@@ -2641,13 +2700,13 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B72" t="s">
         <v>8</v>
       </c>
       <c r="C72" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D72">
         <v>6</v>
@@ -2664,13 +2723,13 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B73" t="s">
         <v>8</v>
       </c>
       <c r="C73" t="s">
-        <v>217</v>
+        <v>116</v>
       </c>
       <c r="D73">
         <v>10</v>
@@ -2687,12 +2746,11 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B74" t="s">
-        <v>136</v>
-      </c>
-      <c r="C74"/>
+        <v>137</v>
+      </c>
       <c r="D74">
         <v>11</v>
       </c>
@@ -2703,18 +2761,18 @@
         <v>21</v>
       </c>
       <c r="G74" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B75" t="s">
         <v>8</v>
       </c>
       <c r="C75" t="s">
-        <v>220</v>
+        <v>119</v>
       </c>
       <c r="D75">
         <v>10</v>
@@ -2731,10 +2789,10 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B76" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C76" t="s">
         <v>122</v>
@@ -2754,7 +2812,7 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B77" t="s">
         <v>8</v>
@@ -2777,13 +2835,13 @@
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A78" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B78" t="s">
         <v>8</v>
       </c>
       <c r="C78" t="s">
-        <v>218</v>
+        <v>142</v>
       </c>
       <c r="D78">
         <v>10</v>
@@ -2800,12 +2858,11 @@
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B79" t="s">
         <v>29</v>
       </c>
-      <c r="C79"/>
       <c r="D79">
         <v>12</v>
       </c>
@@ -2821,7 +2878,7 @@
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B80" t="s">
         <v>8</v>
@@ -2844,13 +2901,13 @@
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B81" t="s">
         <v>8</v>
       </c>
       <c r="C81" t="s">
-        <v>222</v>
+        <v>146</v>
       </c>
       <c r="D81">
         <v>10</v>
@@ -2867,7 +2924,7 @@
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B82" t="s">
         <v>8</v>
@@ -2890,13 +2947,13 @@
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B83" t="s">
         <v>8</v>
       </c>
       <c r="C83" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D83">
         <v>10</v>
@@ -2913,7 +2970,7 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B84" t="s">
         <v>8</v>
@@ -2936,13 +2993,13 @@
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B85" t="s">
         <v>8</v>
       </c>
       <c r="C85" t="s">
-        <v>219</v>
+        <v>151</v>
       </c>
       <c r="D85">
         <v>10</v>
@@ -2959,13 +3016,13 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B86" t="s">
         <v>8</v>
       </c>
       <c r="C86" t="s">
-        <v>220</v>
+        <v>119</v>
       </c>
       <c r="D86">
         <v>10</v>
@@ -2982,7 +3039,7 @@
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B87" t="s">
         <v>8</v>
@@ -3005,12 +3062,11 @@
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B88" t="s">
         <v>8</v>
       </c>
-      <c r="C88"/>
       <c r="D88">
         <v>10</v>
       </c>
@@ -3026,13 +3082,13 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B89" t="s">
         <v>8</v>
       </c>
       <c r="C89" t="s">
-        <v>223</v>
+        <v>156</v>
       </c>
       <c r="D89">
         <v>10</v>
@@ -3049,12 +3105,11 @@
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B90" t="s">
-        <v>153</v>
-      </c>
-      <c r="C90"/>
+        <v>158</v>
+      </c>
       <c r="D90">
         <v>11</v>
       </c>
@@ -3070,12 +3125,11 @@
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B91" t="s">
         <v>8</v>
       </c>
-      <c r="C91"/>
       <c r="D91">
         <v>10</v>
       </c>
@@ -3091,13 +3145,13 @@
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B92" t="s">
         <v>8</v>
       </c>
       <c r="C92" t="s">
-        <v>220</v>
+        <v>119</v>
       </c>
       <c r="D92">
         <v>10</v>
@@ -3114,13 +3168,13 @@
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B93" t="s">
         <v>8</v>
       </c>
       <c r="C93" t="s">
-        <v>224</v>
+        <v>162</v>
       </c>
       <c r="D93">
         <v>10</v>
@@ -3137,7 +3191,7 @@
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B94" t="s">
         <v>8</v>
@@ -3160,13 +3214,13 @@
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B95" t="s">
         <v>8</v>
       </c>
       <c r="C95" t="s">
-        <v>225</v>
+        <v>165</v>
       </c>
       <c r="D95">
         <v>10</v>
@@ -3183,13 +3237,13 @@
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A96" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B96" t="s">
         <v>8</v>
       </c>
       <c r="C96" t="s">
-        <v>226</v>
+        <v>167</v>
       </c>
       <c r="D96">
         <v>6</v>
@@ -3206,13 +3260,13 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B97" t="s">
         <v>8</v>
       </c>
       <c r="C97" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="D97">
         <v>10</v>
@@ -3229,12 +3283,11 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B98" t="s">
         <v>43</v>
       </c>
-      <c r="C98"/>
       <c r="D98">
         <v>11</v>
       </c>
@@ -3250,13 +3303,13 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A99" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B99" t="s">
         <v>8</v>
       </c>
       <c r="C99" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="D99">
         <v>10</v>
@@ -3273,13 +3326,13 @@
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A100" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B100" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="C100" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="D100">
         <v>11</v>
@@ -3296,7 +3349,7 @@
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A101" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="B101" t="s">
         <v>8</v>
@@ -3319,7 +3372,7 @@
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A102" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B102" t="s">
         <v>8</v>
@@ -3342,12 +3395,11 @@
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="B103" t="s">
-        <v>171</v>
-      </c>
-      <c r="C103"/>
+        <v>179</v>
+      </c>
       <c r="D103">
         <v>11</v>
       </c>
@@ -3363,13 +3415,13 @@
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A104" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="B104" t="s">
         <v>8</v>
       </c>
       <c r="C104" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D104">
         <v>10</v>
@@ -3386,13 +3438,13 @@
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A105" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B105" t="s">
         <v>8</v>
       </c>
       <c r="C105" t="s">
-        <v>217</v>
+        <v>116</v>
       </c>
       <c r="D105">
         <v>10</v>
@@ -3409,10 +3461,10 @@
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A106" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="B106" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C106" t="s">
         <v>122</v>
@@ -3432,13 +3484,13 @@
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A107" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B107" t="s">
         <v>8</v>
       </c>
       <c r="C107" t="s">
-        <v>227</v>
+        <v>184</v>
       </c>
       <c r="D107">
         <v>6</v>
@@ -3455,13 +3507,13 @@
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="B108" t="s">
         <v>8</v>
       </c>
       <c r="C108" t="s">
-        <v>228</v>
+        <v>186</v>
       </c>
       <c r="D108">
         <v>10</v>
@@ -3473,18 +3525,18 @@
         <v>21</v>
       </c>
       <c r="G108" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A109" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="B109" t="s">
         <v>8</v>
       </c>
       <c r="C109" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="D109">
         <v>10</v>
@@ -3501,13 +3553,13 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A110" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="B110" t="s">
         <v>8</v>
       </c>
       <c r="C110" t="s">
-        <v>229</v>
+        <v>190</v>
       </c>
       <c r="D110">
         <v>10</v>
@@ -3519,12 +3571,12 @@
         <v>21</v>
       </c>
       <c r="G110" t="s">
-        <v>230</v>
+        <v>191</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A111" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="B111" t="s">
         <v>8</v>
@@ -3547,12 +3599,11 @@
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="B112" t="s">
         <v>43</v>
       </c>
-      <c r="C112"/>
       <c r="D112">
         <v>11</v>
       </c>
@@ -3568,10 +3619,10 @@
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A113" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="B113" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C113" t="s">
         <v>122</v>
@@ -3591,7 +3642,7 @@
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A114" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="B114" t="s">
         <v>8</v>
@@ -3614,13 +3665,13 @@
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A115" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="B115" t="s">
         <v>8</v>
       </c>
       <c r="C115" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="D115">
         <v>10</v>
@@ -3632,18 +3683,18 @@
         <v>21</v>
       </c>
       <c r="G115" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A116" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="B116" t="s">
         <v>8</v>
       </c>
       <c r="C116" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="D116">
         <v>10</v>
@@ -3660,13 +3711,13 @@
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A117" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="B117" t="s">
         <v>8</v>
       </c>
       <c r="C117" t="s">
-        <v>228</v>
+        <v>186</v>
       </c>
       <c r="D117">
         <v>10</v>
@@ -3683,13 +3734,13 @@
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A118" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="B118" t="s">
         <v>8</v>
       </c>
       <c r="C118" t="s">
-        <v>228</v>
+        <v>186</v>
       </c>
       <c r="D118">
         <v>10</v>
@@ -3706,7 +3757,7 @@
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A119" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="B119" t="s">
         <v>8</v>
@@ -3729,13 +3780,13 @@
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A120" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="B120" t="s">
         <v>58</v>
       </c>
       <c r="C120" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="D120">
         <v>10</v>
@@ -3752,7 +3803,7 @@
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A121" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="B121" t="s">
         <v>8</v>
@@ -3775,13 +3826,13 @@
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A122" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="B122" t="s">
         <v>8</v>
       </c>
       <c r="C122" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="D122">
         <v>11</v>
@@ -3793,12 +3844,12 @@
         <v>21</v>
       </c>
       <c r="G122" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A123" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="B123" t="s">
         <v>8</v>
@@ -3816,18 +3867,18 @@
         <v>21</v>
       </c>
       <c r="G123" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A124" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="B124" t="s">
         <v>8</v>
       </c>
       <c r="C124" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="D124">
         <v>10</v>
@@ -3844,7 +3895,7 @@
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A125" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="B125" t="s">
         <v>8</v>
@@ -3867,13 +3918,13 @@
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A126" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="B126" t="s">
         <v>8</v>
       </c>
       <c r="C126" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="D126">
         <v>10</v>
@@ -3890,13 +3941,13 @@
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A127" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="B127" t="s">
         <v>8</v>
       </c>
       <c r="C127" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D127">
         <v>10</v>
@@ -3913,13 +3964,13 @@
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A128" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="B128" t="s">
         <v>8</v>
       </c>
       <c r="C128" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D128">
         <v>10</v>
@@ -3936,7 +3987,7 @@
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A129" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="B129" t="s">
         <v>8</v>
@@ -3959,13 +4010,13 @@
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A130" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="B130" t="s">
         <v>8</v>
       </c>
       <c r="C130" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D130">
         <v>10</v>
@@ -3982,7 +4033,7 @@
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A131" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="B131" t="s">
         <v>8</v>
@@ -4005,12 +4056,11 @@
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A132" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="B132" t="s">
-        <v>153</v>
-      </c>
-      <c r="C132"/>
+        <v>158</v>
+      </c>
       <c r="D132">
         <v>11</v>
       </c>
@@ -4026,13 +4076,13 @@
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A133" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B133" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="C133" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="D133">
         <v>11</v>
@@ -4049,7 +4099,7 @@
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A134" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="B134" t="s">
         <v>8</v>
@@ -4072,13 +4122,13 @@
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A135" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="B135" t="s">
         <v>8</v>
       </c>
       <c r="C135" t="s">
-        <v>117</v>
+        <v>218</v>
       </c>
       <c r="D135">
         <v>10</v>
@@ -4090,17 +4140,16 @@
         <v>21</v>
       </c>
       <c r="G135" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A136" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="B136" t="s">
-        <v>153</v>
-      </c>
-      <c r="C136"/>
+        <v>158</v>
+      </c>
       <c r="D136">
         <v>11</v>
       </c>
@@ -4116,12 +4165,11 @@
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A137" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="B137" t="s">
         <v>43</v>
       </c>
-      <c r="C137"/>
       <c r="D137">
         <v>11</v>
       </c>
@@ -4137,12 +4185,11 @@
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A138" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="B138" t="s">
-        <v>209</v>
-      </c>
-      <c r="C138"/>
+        <v>222</v>
+      </c>
       <c r="D138">
         <v>11</v>
       </c>
@@ -4158,22 +4205,22 @@
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A139" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="B139" t="s">
         <v>8</v>
       </c>
       <c r="C139" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="D139">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="E139">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F139" t="s">
-        <v>21</v>
+        <v>225</v>
       </c>
       <c r="G139" t="s">
         <v>11</v>
@@ -4181,12 +4228,11 @@
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A140" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="B140" t="s">
         <v>43</v>
       </c>
-      <c r="C140"/>
       <c r="D140">
         <v>11</v>
       </c>
@@ -4202,13 +4248,13 @@
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A141" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="B141" t="s">
         <v>8</v>
       </c>
       <c r="C141" t="s">
-        <v>225</v>
+        <v>165</v>
       </c>
       <c r="D141">
         <v>10</v>
@@ -4225,7 +4271,7 @@
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A142" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="B142" t="s">
         <v>8</v>
@@ -4248,13 +4294,13 @@
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A143" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B143" t="s">
         <v>8</v>
       </c>
       <c r="C143" t="s">
-        <v>220</v>
+        <v>119</v>
       </c>
       <c r="D143">
         <v>10</v>
@@ -4271,13 +4317,13 @@
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A144" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="B144" t="s">
         <v>8</v>
       </c>
       <c r="C144" t="s">
-        <v>220</v>
+        <v>119</v>
       </c>
       <c r="D144">
         <v>11</v>
@@ -4290,6 +4336,305 @@
       </c>
       <c r="G144" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A145" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="D145" s="1">
+        <v>6</v>
+      </c>
+      <c r="E145" s="1">
+        <v>14</v>
+      </c>
+      <c r="F145" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G145" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A146" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B146" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="D146" s="1">
+        <v>11</v>
+      </c>
+      <c r="E146" s="1">
+        <v>0</v>
+      </c>
+      <c r="F146" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G146" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A147" t="s">
+        <v>235</v>
+      </c>
+      <c r="B147" t="s">
+        <v>8</v>
+      </c>
+      <c r="C147" t="s">
+        <v>232</v>
+      </c>
+      <c r="D147">
+        <v>10</v>
+      </c>
+      <c r="E147">
+        <v>20</v>
+      </c>
+      <c r="F147" t="s">
+        <v>21</v>
+      </c>
+      <c r="G147" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A148" t="s">
+        <v>236</v>
+      </c>
+      <c r="B148" t="s">
+        <v>8</v>
+      </c>
+      <c r="C148" t="s">
+        <v>232</v>
+      </c>
+      <c r="D148">
+        <v>11</v>
+      </c>
+      <c r="E148">
+        <v>20</v>
+      </c>
+      <c r="F148" t="s">
+        <v>21</v>
+      </c>
+      <c r="G148" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A149" t="s">
+        <v>237</v>
+      </c>
+      <c r="B149" t="s">
+        <v>8</v>
+      </c>
+      <c r="C149" t="s">
+        <v>232</v>
+      </c>
+      <c r="D149">
+        <v>6</v>
+      </c>
+      <c r="E149">
+        <v>15</v>
+      </c>
+      <c r="F149" t="s">
+        <v>21</v>
+      </c>
+      <c r="G149" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A150" t="s">
+        <v>238</v>
+      </c>
+      <c r="B150" t="s">
+        <v>8</v>
+      </c>
+      <c r="C150" t="s">
+        <v>239</v>
+      </c>
+      <c r="D150">
+        <v>8</v>
+      </c>
+      <c r="E150">
+        <v>20</v>
+      </c>
+      <c r="F150" t="s">
+        <v>14</v>
+      </c>
+      <c r="G150" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A151" t="s">
+        <v>240</v>
+      </c>
+      <c r="B151" t="s">
+        <v>8</v>
+      </c>
+      <c r="C151" t="s">
+        <v>232</v>
+      </c>
+      <c r="D151">
+        <v>7</v>
+      </c>
+      <c r="E151">
+        <v>15</v>
+      </c>
+      <c r="F151" t="s">
+        <v>225</v>
+      </c>
+      <c r="G151" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A152" t="s">
+        <v>241</v>
+      </c>
+      <c r="B152" t="s">
+        <v>8</v>
+      </c>
+      <c r="C152" t="s">
+        <v>242</v>
+      </c>
+      <c r="D152">
+        <v>8</v>
+      </c>
+      <c r="E152">
+        <v>17</v>
+      </c>
+      <c r="F152" t="s">
+        <v>243</v>
+      </c>
+      <c r="G152" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A153" t="s">
+        <v>244</v>
+      </c>
+      <c r="B153" t="s">
+        <v>8</v>
+      </c>
+      <c r="C153" t="s">
+        <v>232</v>
+      </c>
+      <c r="D153">
+        <v>7</v>
+      </c>
+      <c r="E153">
+        <v>14</v>
+      </c>
+      <c r="F153" t="s">
+        <v>225</v>
+      </c>
+      <c r="G153" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A154" t="s">
+        <v>245</v>
+      </c>
+      <c r="B154" t="s">
+        <v>8</v>
+      </c>
+      <c r="C154" t="s">
+        <v>232</v>
+      </c>
+      <c r="D154">
+        <v>10</v>
+      </c>
+      <c r="E154">
+        <v>22</v>
+      </c>
+      <c r="F154" t="s">
+        <v>246</v>
+      </c>
+      <c r="G154" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A155" t="s">
+        <v>247</v>
+      </c>
+      <c r="B155" t="s">
+        <v>8</v>
+      </c>
+      <c r="C155" t="s">
+        <v>232</v>
+      </c>
+      <c r="D155">
+        <v>10</v>
+      </c>
+      <c r="E155">
+        <v>21</v>
+      </c>
+      <c r="F155" t="s">
+        <v>248</v>
+      </c>
+      <c r="G155" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A156" t="s">
+        <v>249</v>
+      </c>
+      <c r="B156" t="s">
+        <v>8</v>
+      </c>
+      <c r="C156" t="s">
+        <v>232</v>
+      </c>
+      <c r="D156">
+        <v>10</v>
+      </c>
+      <c r="E156">
+        <v>21</v>
+      </c>
+      <c r="F156" t="s">
+        <v>21</v>
+      </c>
+      <c r="G156" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A157" t="s">
+        <v>250</v>
+      </c>
+      <c r="B157" t="s">
+        <v>8</v>
+      </c>
+      <c r="C157" t="s">
+        <v>232</v>
+      </c>
+      <c r="D157">
+        <v>11</v>
+      </c>
+      <c r="E157">
+        <v>22</v>
+      </c>
+      <c r="F157" t="s">
+        <v>18</v>
+      </c>
+      <c r="G157" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove extra mee hoon kueh spots and correct hours in the shared list.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\OneDrive\Documents\Cursor Projects\food-spot-selector\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5FC7E4-DC8B-4607-BE6A-1BD2EC185A3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27CCB027-9262-4863-8622-E7BEF413AF08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="12549" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="246">
   <si>
     <t>Place</t>
   </si>
@@ -727,12 +727,6 @@
     <t>Beef Kway Teow, Noodles</t>
   </si>
   <si>
-    <t>Greenview Cafe</t>
-  </si>
-  <si>
-    <t>Madam Tyrant</t>
-  </si>
-  <si>
     <t>Seletar Sheng Mian &amp; Mian Fen Guo</t>
   </si>
   <si>
@@ -742,9 +736,6 @@
     <t>Mee Hoon Kueh, Fish Soup, Noodles</t>
   </si>
   <si>
-    <t>Ai Chi Mee Hoon Kueh</t>
-  </si>
-  <si>
     <t>Banting Traditional Cuisine</t>
   </si>
   <si>
@@ -763,16 +754,10 @@
     <t>Fri</t>
   </si>
   <si>
-    <t>Penang Heng Heng Handmade Noodle</t>
-  </si>
-  <si>
-    <t>Tue</t>
-  </si>
-  <si>
-    <t>Jiak Song Mee Hoon Kway</t>
-  </si>
-  <si>
     <t>L32 Handmade Noodles</t>
+  </si>
+  <si>
+    <t>Mee Hoon Kueh, Ban Mian, Noodles</t>
   </si>
 </sst>
 </file>
@@ -1096,18 +1081,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H157"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:H152"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.921875" style="1" customWidth="1"/>
-    <col min="2" max="3" width="29.69140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.90625" style="1" customWidth="1"/>
+    <col min="2" max="3" width="29.7265625" style="1" customWidth="1"/>
     <col min="4" max="4" width="21" style="1" customWidth="1"/>
-    <col min="5" max="6" width="15.15234375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.4609375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="27.61328125" style="1" customWidth="1"/>
+    <col min="5" max="6" width="15.1796875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.453125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="27.6328125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1130,7 +1115,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1153,7 +1138,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1176,7 +1161,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -1199,7 +1184,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -1222,7 +1207,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="58.3" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="58.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
@@ -1245,7 +1230,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
@@ -1268,7 +1253,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>25</v>
       </c>
@@ -1291,7 +1276,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
@@ -1314,7 +1299,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
@@ -1337,7 +1322,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>28</v>
       </c>
@@ -1360,7 +1345,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>31</v>
       </c>
@@ -1383,7 +1368,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>33</v>
       </c>
@@ -1406,7 +1391,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>35</v>
       </c>
@@ -1426,7 +1411,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>37</v>
       </c>
@@ -1446,7 +1431,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>38</v>
       </c>
@@ -1466,7 +1451,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>39</v>
       </c>
@@ -1489,7 +1474,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>42</v>
       </c>
@@ -1509,7 +1494,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>45</v>
       </c>
@@ -1532,7 +1517,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>46</v>
       </c>
@@ -1552,7 +1537,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>47</v>
       </c>
@@ -1575,7 +1560,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>48</v>
       </c>
@@ -1598,7 +1583,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>52</v>
       </c>
@@ -1618,7 +1603,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>53</v>
       </c>
@@ -1641,7 +1626,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>56</v>
       </c>
@@ -1661,7 +1646,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>57</v>
       </c>
@@ -1684,7 +1669,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>60</v>
       </c>
@@ -1707,7 +1692,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>61</v>
       </c>
@@ -1730,7 +1715,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>64</v>
       </c>
@@ -1753,7 +1738,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>66</v>
       </c>
@@ -1773,7 +1758,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="43.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:7" ht="43.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>68</v>
       </c>
@@ -1796,7 +1781,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>69</v>
       </c>
@@ -1819,7 +1804,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>71</v>
       </c>
@@ -1842,7 +1827,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>72</v>
       </c>
@@ -1865,7 +1850,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>74</v>
       </c>
@@ -1888,7 +1873,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>76</v>
       </c>
@@ -1911,7 +1896,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>77</v>
       </c>
@@ -1934,7 +1919,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>78</v>
       </c>
@@ -1954,7 +1939,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>81</v>
       </c>
@@ -1974,7 +1959,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>82</v>
       </c>
@@ -1994,7 +1979,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>83</v>
       </c>
@@ -2017,7 +2002,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>86</v>
       </c>
@@ -2037,7 +2022,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>87</v>
       </c>
@@ -2060,7 +2045,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>89</v>
       </c>
@@ -2083,7 +2068,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>91</v>
       </c>
@@ -2106,7 +2091,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>92</v>
       </c>
@@ -2126,7 +2111,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>93</v>
       </c>
@@ -2149,7 +2134,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>95</v>
       </c>
@@ -2172,7 +2157,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>96</v>
       </c>
@@ -2195,7 +2180,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>98</v>
       </c>
@@ -2218,7 +2203,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>99</v>
       </c>
@@ -2241,7 +2226,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>102</v>
       </c>
@@ -2264,7 +2249,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>104</v>
       </c>
@@ -2287,7 +2272,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>106</v>
       </c>
@@ -2310,7 +2295,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>110</v>
       </c>
@@ -2333,7 +2318,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>111</v>
       </c>
@@ -2356,7 +2341,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>112</v>
       </c>
@@ -2376,7 +2361,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>113</v>
       </c>
@@ -2399,7 +2384,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>115</v>
       </c>
@@ -2422,7 +2407,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>117</v>
       </c>
@@ -2445,7 +2430,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>118</v>
       </c>
@@ -2468,7 +2453,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>120</v>
       </c>
@@ -2491,7 +2476,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>121</v>
       </c>
@@ -2514,7 +2499,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>123</v>
       </c>
@@ -2537,7 +2522,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>124</v>
       </c>
@@ -2560,7 +2545,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>125</v>
       </c>
@@ -2583,7 +2568,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>126</v>
       </c>
@@ -2606,7 +2591,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>128</v>
       </c>
@@ -2629,7 +2614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>129</v>
       </c>
@@ -2652,7 +2637,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>130</v>
       </c>
@@ -2675,7 +2660,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>132</v>
       </c>
@@ -2698,7 +2683,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>133</v>
       </c>
@@ -2721,7 +2706,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>135</v>
       </c>
@@ -2744,7 +2729,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>136</v>
       </c>
@@ -2764,7 +2749,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>138</v>
       </c>
@@ -2787,7 +2772,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>139</v>
       </c>
@@ -2810,7 +2795,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>140</v>
       </c>
@@ -2833,7 +2818,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>141</v>
       </c>
@@ -2856,7 +2841,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>143</v>
       </c>
@@ -2876,7 +2861,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>144</v>
       </c>
@@ -2899,7 +2884,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>145</v>
       </c>
@@ -2922,7 +2907,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>147</v>
       </c>
@@ -2945,7 +2930,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>148</v>
       </c>
@@ -2968,7 +2953,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>149</v>
       </c>
@@ -2991,7 +2976,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>150</v>
       </c>
@@ -3014,7 +2999,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>152</v>
       </c>
@@ -3037,7 +3022,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>153</v>
       </c>
@@ -3060,7 +3045,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>154</v>
       </c>
@@ -3080,7 +3065,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>155</v>
       </c>
@@ -3103,7 +3088,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>157</v>
       </c>
@@ -3123,7 +3108,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>159</v>
       </c>
@@ -3143,7 +3128,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>160</v>
       </c>
@@ -3166,7 +3151,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>161</v>
       </c>
@@ -3189,7 +3174,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>163</v>
       </c>
@@ -3212,7 +3197,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>164</v>
       </c>
@@ -3235,7 +3220,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>166</v>
       </c>
@@ -3258,7 +3243,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>168</v>
       </c>
@@ -3281,7 +3266,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>170</v>
       </c>
@@ -3301,7 +3286,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>171</v>
       </c>
@@ -3324,7 +3309,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>173</v>
       </c>
@@ -3347,7 +3332,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>176</v>
       </c>
@@ -3370,7 +3355,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>177</v>
       </c>
@@ -3393,7 +3378,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>178</v>
       </c>
@@ -3413,7 +3398,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>180</v>
       </c>
@@ -3436,7 +3421,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>181</v>
       </c>
@@ -3459,7 +3444,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>182</v>
       </c>
@@ -3482,7 +3467,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>183</v>
       </c>
@@ -3505,7 +3490,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>185</v>
       </c>
@@ -3528,7 +3513,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>187</v>
       </c>
@@ -3551,7 +3536,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>189</v>
       </c>
@@ -3574,7 +3559,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>192</v>
       </c>
@@ -3597,7 +3582,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>193</v>
       </c>
@@ -3617,7 +3602,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>194</v>
       </c>
@@ -3640,7 +3625,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>195</v>
       </c>
@@ -3663,7 +3648,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>196</v>
       </c>
@@ -3686,7 +3671,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>198</v>
       </c>
@@ -3709,7 +3694,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>199</v>
       </c>
@@ -3732,7 +3717,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>200</v>
       </c>
@@ -3755,7 +3740,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>201</v>
       </c>
@@ -3778,7 +3763,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>202</v>
       </c>
@@ -3801,7 +3786,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>203</v>
       </c>
@@ -3824,7 +3809,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>204</v>
       </c>
@@ -3847,7 +3832,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>205</v>
       </c>
@@ -3870,7 +3855,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>206</v>
       </c>
@@ -3893,7 +3878,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>207</v>
       </c>
@@ -3916,7 +3901,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>208</v>
       </c>
@@ -3939,7 +3924,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>209</v>
       </c>
@@ -3962,7 +3947,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>210</v>
       </c>
@@ -3985,7 +3970,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>211</v>
       </c>
@@ -4008,7 +3993,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>212</v>
       </c>
@@ -4031,7 +4016,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>213</v>
       </c>
@@ -4054,7 +4039,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>214</v>
       </c>
@@ -4074,7 +4059,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>215</v>
       </c>
@@ -4097,7 +4082,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>216</v>
       </c>
@@ -4120,7 +4105,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>217</v>
       </c>
@@ -4143,7 +4128,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>219</v>
       </c>
@@ -4163,7 +4148,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>220</v>
       </c>
@@ -4183,7 +4168,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>221</v>
       </c>
@@ -4203,7 +4188,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>223</v>
       </c>
@@ -4226,7 +4211,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>226</v>
       </c>
@@ -4246,7 +4231,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>227</v>
       </c>
@@ -4269,7 +4254,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>228</v>
       </c>
@@ -4292,7 +4277,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>229</v>
       </c>
@@ -4315,7 +4300,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>230</v>
       </c>
@@ -4338,7 +4323,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="145" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="145" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>231</v>
       </c>
@@ -4361,7 +4346,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="146" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="146" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>233</v>
       </c>
@@ -4384,7 +4369,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>235</v>
       </c>
@@ -4395,19 +4380,19 @@
         <v>232</v>
       </c>
       <c r="D147">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E147">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F147" t="s">
-        <v>21</v>
+        <v>243</v>
       </c>
       <c r="G147" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>236</v>
       </c>
@@ -4415,225 +4400,110 @@
         <v>8</v>
       </c>
       <c r="C148" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="D148">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E148">
         <v>20</v>
       </c>
       <c r="F148" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G148" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.4">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B149" t="s">
         <v>8</v>
       </c>
       <c r="C149" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="D149">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E149">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F149" t="s">
-        <v>21</v>
+        <v>240</v>
       </c>
       <c r="G149" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B150" t="s">
         <v>8</v>
       </c>
       <c r="C150" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="D150">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E150">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F150" t="s">
-        <v>14</v>
+        <v>240</v>
       </c>
       <c r="G150" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
+        <v>242</v>
+      </c>
+      <c r="B151" t="s">
+        <v>8</v>
+      </c>
+      <c r="C151" t="s">
+        <v>245</v>
+      </c>
+      <c r="D151">
+        <v>8</v>
+      </c>
+      <c r="E151">
+        <v>23</v>
+      </c>
+      <c r="F151" t="s">
         <v>240</v>
       </c>
-      <c r="B151" t="s">
-        <v>8</v>
-      </c>
-      <c r="C151" t="s">
-        <v>232</v>
-      </c>
-      <c r="D151">
-        <v>7</v>
-      </c>
-      <c r="E151">
-        <v>15</v>
-      </c>
-      <c r="F151" t="s">
-        <v>225</v>
-      </c>
       <c r="G151" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B152" t="s">
         <v>8</v>
       </c>
       <c r="C152" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D152">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E152">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F152" t="s">
-        <v>243</v>
+        <v>18</v>
       </c>
       <c r="G152" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A153" t="s">
-        <v>244</v>
-      </c>
-      <c r="B153" t="s">
-        <v>8</v>
-      </c>
-      <c r="C153" t="s">
-        <v>232</v>
-      </c>
-      <c r="D153">
-        <v>7</v>
-      </c>
-      <c r="E153">
-        <v>14</v>
-      </c>
-      <c r="F153" t="s">
-        <v>225</v>
-      </c>
-      <c r="G153" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A154" t="s">
-        <v>245</v>
-      </c>
-      <c r="B154" t="s">
-        <v>8</v>
-      </c>
-      <c r="C154" t="s">
-        <v>232</v>
-      </c>
-      <c r="D154">
-        <v>10</v>
-      </c>
-      <c r="E154">
-        <v>22</v>
-      </c>
-      <c r="F154" t="s">
-        <v>246</v>
-      </c>
-      <c r="G154" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A155" t="s">
-        <v>247</v>
-      </c>
-      <c r="B155" t="s">
-        <v>8</v>
-      </c>
-      <c r="C155" t="s">
-        <v>232</v>
-      </c>
-      <c r="D155">
-        <v>10</v>
-      </c>
-      <c r="E155">
-        <v>21</v>
-      </c>
-      <c r="F155" t="s">
-        <v>248</v>
-      </c>
-      <c r="G155" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A156" t="s">
-        <v>249</v>
-      </c>
-      <c r="B156" t="s">
-        <v>8</v>
-      </c>
-      <c r="C156" t="s">
-        <v>232</v>
-      </c>
-      <c r="D156">
-        <v>10</v>
-      </c>
-      <c r="E156">
-        <v>21</v>
-      </c>
-      <c r="F156" t="s">
-        <v>21</v>
-      </c>
-      <c r="G156" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A157" t="s">
-        <v>250</v>
-      </c>
-      <c r="B157" t="s">
-        <v>8</v>
-      </c>
-      <c r="C157" t="s">
-        <v>232</v>
-      </c>
-      <c r="D157">
-        <v>11</v>
-      </c>
-      <c r="E157">
-        <v>22</v>
-      </c>
-      <c r="F157" t="s">
-        <v>18</v>
-      </c>
-      <c r="G157" t="s">
         <v>70</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct hours, closing days, and tags in the shared list.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27CCB027-9262-4863-8622-E7BEF413AF08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24CED9D4-3D99-4583-B8FB-1CCE2F2E09D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="249">
   <si>
     <t>Place</t>
   </si>
@@ -758,6 +758,15 @@
   </si>
   <si>
     <t>Mee Hoon Kueh, Ban Mian, Noodles</t>
+  </si>
+  <si>
+    <t>North, East</t>
+  </si>
+  <si>
+    <t>Wed, Thu</t>
+  </si>
+  <si>
+    <t>Soup, Biryani</t>
   </si>
 </sst>
 </file>
@@ -1534,7 +1543,7 @@
         <v>21</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>11</v>
+        <v>246</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -2510,13 +2519,13 @@
         <v>20</v>
       </c>
       <c r="D64">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E64">
         <v>20</v>
       </c>
       <c r="F64" t="s">
-        <v>21</v>
+        <v>240</v>
       </c>
       <c r="G64" t="s">
         <v>11</v>
@@ -2530,13 +2539,13 @@
         <v>107</v>
       </c>
       <c r="C65" t="s">
-        <v>20</v>
+        <v>248</v>
       </c>
       <c r="D65">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E65">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F65" t="s">
         <v>21</v>
@@ -2556,10 +2565,10 @@
         <v>84</v>
       </c>
       <c r="D66">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E66">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F66" t="s">
         <v>21</v>
@@ -2829,10 +2838,10 @@
         <v>142</v>
       </c>
       <c r="D78">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E78">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F78" t="s">
         <v>21</v>
@@ -2872,13 +2881,13 @@
         <v>73</v>
       </c>
       <c r="D80">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E80">
         <v>20</v>
       </c>
       <c r="F80" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G80" t="s">
         <v>11</v>
@@ -2895,13 +2904,13 @@
         <v>146</v>
       </c>
       <c r="D81">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E81">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F81" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G81" t="s">
         <v>11</v>
@@ -2918,10 +2927,10 @@
         <v>17</v>
       </c>
       <c r="D82">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E82">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F82" t="s">
         <v>21</v>
@@ -2941,10 +2950,10 @@
         <v>84</v>
       </c>
       <c r="D83">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E83">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F83" t="s">
         <v>21</v>
@@ -2964,13 +2973,13 @@
         <v>73</v>
       </c>
       <c r="D84">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E84">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F84" t="s">
-        <v>21</v>
+        <v>247</v>
       </c>
       <c r="G84" t="s">
         <v>15</v>
@@ -2990,10 +2999,10 @@
         <v>10</v>
       </c>
       <c r="E85">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F85" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="G85" t="s">
         <v>11</v>
@@ -3013,10 +3022,10 @@
         <v>10</v>
       </c>
       <c r="E86">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F86" t="s">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="G86" t="s">
         <v>11</v>
@@ -3033,13 +3042,13 @@
         <v>20</v>
       </c>
       <c r="D87">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E87">
         <v>20</v>
       </c>
       <c r="F87" t="s">
-        <v>21</v>
+        <v>225</v>
       </c>
       <c r="G87" t="s">
         <v>11</v>
@@ -4265,10 +4274,10 @@
         <v>32</v>
       </c>
       <c r="D142">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E142">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F142" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Update hours, closing days, and tags in the shared list.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\Projects\food-spot-selector\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\OneDrive\Documents\Cursor Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24CED9D4-3D99-4583-B8FB-1CCE2F2E09D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F36AB3C-3077-48A3-BF34-1A0C74A95629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10886" yWindow="0" windowWidth="11143" windowHeight="12429" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="260">
   <si>
     <t>Place</t>
   </si>
@@ -538,9 +538,6 @@
     <t>Kelantan Kway Chap · Pig Organ Soup</t>
   </si>
   <si>
-    <t>Kway Chap, Soup</t>
-  </si>
-  <si>
     <t>Kitchenman Nasi Lemak</t>
   </si>
   <si>
@@ -595,9 +592,6 @@
     <t>Fishball Noodles, Noodles</t>
   </si>
   <si>
-    <t>North, East, Central, West</t>
-  </si>
-  <si>
     <t>Margaret Drive Sin Kee Chicken Rice</t>
   </si>
   <si>
@@ -655,9 +649,6 @@
     <t>Song Kee Teochew Fish Porridge</t>
   </si>
   <si>
-    <t>Spinach Soup</t>
-  </si>
-  <si>
     <t>Tai Seng Fish Soup</t>
   </si>
   <si>
@@ -673,12 +664,6 @@
     <t>Tiong Bahru Hainanese Boneless Chicken Rice</t>
   </si>
   <si>
-    <t>To-Ricos Kway Chap</t>
-  </si>
-  <si>
-    <t>Kway Chap</t>
-  </si>
-  <si>
     <t>True Blue Cuisine</t>
   </si>
   <si>
@@ -767,6 +752,54 @@
   </si>
   <si>
     <t>Soup, Biryani</t>
+  </si>
+  <si>
+    <t>Thu, Fri</t>
+  </si>
+  <si>
+    <t>Fri, Mon</t>
+  </si>
+  <si>
+    <t>Italian</t>
+  </si>
+  <si>
+    <t>Mon, Tue</t>
+  </si>
+  <si>
+    <t>Sat, Sun, Mon</t>
+  </si>
+  <si>
+    <t>Curry Puff</t>
+  </si>
+  <si>
+    <t>Tue</t>
+  </si>
+  <si>
+    <t>Kway Chap, Pig Organ Soup, Soup</t>
+  </si>
+  <si>
+    <t>Pig Organ Soup, Soup</t>
+  </si>
+  <si>
+    <t>Fish Soup, Soup</t>
+  </si>
+  <si>
+    <t>Wed, Sun</t>
+  </si>
+  <si>
+    <t>Mon, Thu</t>
+  </si>
+  <si>
+    <t>Mee Rebus, Mee Soto, Noodles</t>
+  </si>
+  <si>
+    <t>Seafood, Tze Char</t>
+  </si>
+  <si>
+    <t>Yuan Yang Spinach Soup</t>
+  </si>
+  <si>
+    <t>Prawn Noodles, Hokkien Mee, Noodles</t>
   </si>
 </sst>
 </file>
@@ -1090,18 +1123,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H152"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H151"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.90625" style="1" customWidth="1"/>
-    <col min="2" max="3" width="29.7265625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.921875" style="1" customWidth="1"/>
+    <col min="2" max="3" width="29.69140625" style="1" customWidth="1"/>
     <col min="4" max="4" width="21" style="1" customWidth="1"/>
-    <col min="5" max="6" width="15.1796875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.453125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="27.6328125" style="1" customWidth="1"/>
+    <col min="5" max="6" width="15.15234375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.4609375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="27.61328125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1124,7 +1157,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1147,7 +1180,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -1170,7 +1203,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -1193,7 +1226,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -1216,7 +1249,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="58.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="58.3" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
@@ -1239,7 +1272,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
@@ -1262,7 +1295,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>25</v>
       </c>
@@ -1285,7 +1318,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
@@ -1308,7 +1341,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
@@ -1331,7 +1364,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>28</v>
       </c>
@@ -1354,7 +1387,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>31</v>
       </c>
@@ -1377,7 +1410,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
         <v>33</v>
       </c>
@@ -1400,7 +1433,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>35</v>
       </c>
@@ -1420,7 +1453,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>37</v>
       </c>
@@ -1440,7 +1473,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
         <v>38</v>
       </c>
@@ -1460,7 +1493,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
         <v>39</v>
       </c>
@@ -1483,7 +1516,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>42</v>
       </c>
@@ -1503,7 +1536,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
         <v>45</v>
       </c>
@@ -1526,7 +1559,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
         <v>46</v>
       </c>
@@ -1543,10 +1576,10 @@
         <v>21</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
         <v>47</v>
       </c>
@@ -1569,7 +1602,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>48</v>
       </c>
@@ -1592,7 +1625,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
         <v>52</v>
       </c>
@@ -1612,7 +1645,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>53</v>
       </c>
@@ -1635,7 +1668,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
         <v>56</v>
       </c>
@@ -1655,7 +1688,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
         <v>57</v>
       </c>
@@ -1678,7 +1711,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>60</v>
       </c>
@@ -1701,7 +1734,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
         <v>61</v>
       </c>
@@ -1724,7 +1757,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
         <v>64</v>
       </c>
@@ -1747,7 +1780,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>66</v>
       </c>
@@ -1767,7 +1800,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="43.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="43.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>68</v>
       </c>
@@ -1790,7 +1823,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="1" t="s">
         <v>69</v>
       </c>
@@ -1813,7 +1846,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
         <v>71</v>
       </c>
@@ -1836,7 +1869,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
         <v>72</v>
       </c>
@@ -1859,7 +1892,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
         <v>74</v>
       </c>
@@ -1882,7 +1915,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="1" t="s">
         <v>76</v>
       </c>
@@ -1905,7 +1938,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="1" t="s">
         <v>77</v>
       </c>
@@ -1928,7 +1961,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A38" s="1" t="s">
         <v>78</v>
       </c>
@@ -1948,7 +1981,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A39" s="1" t="s">
         <v>81</v>
       </c>
@@ -1968,7 +2001,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
         <v>82</v>
       </c>
@@ -1988,7 +2021,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">
         <v>83</v>
       </c>
@@ -2011,7 +2044,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A42" s="1" t="s">
         <v>86</v>
       </c>
@@ -2031,7 +2064,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A43" s="1" t="s">
         <v>87</v>
       </c>
@@ -2054,7 +2087,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A44" s="1" t="s">
         <v>89</v>
       </c>
@@ -2077,7 +2110,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A45" s="1" t="s">
         <v>91</v>
       </c>
@@ -2100,7 +2133,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A46" s="1" t="s">
         <v>92</v>
       </c>
@@ -2120,7 +2153,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A47" s="1" t="s">
         <v>93</v>
       </c>
@@ -2143,7 +2176,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A48" s="1" t="s">
         <v>95</v>
       </c>
@@ -2166,7 +2199,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>96</v>
       </c>
@@ -2189,7 +2222,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
         <v>98</v>
       </c>
@@ -2212,7 +2245,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
         <v>99</v>
       </c>
@@ -2235,7 +2268,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
         <v>102</v>
       </c>
@@ -2258,7 +2291,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
         <v>104</v>
       </c>
@@ -2281,7 +2314,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
         <v>106</v>
       </c>
@@ -2304,7 +2337,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
         <v>110</v>
       </c>
@@ -2327,7 +2360,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
         <v>111</v>
       </c>
@@ -2350,7 +2383,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
         <v>112</v>
       </c>
@@ -2370,7 +2403,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
         <v>113</v>
       </c>
@@ -2393,7 +2426,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
         <v>115</v>
       </c>
@@ -2416,7 +2449,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
         <v>117</v>
       </c>
@@ -2439,7 +2472,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
         <v>118</v>
       </c>
@@ -2462,7 +2495,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A62" t="s">
         <v>120</v>
       </c>
@@ -2485,7 +2518,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
         <v>121</v>
       </c>
@@ -2508,7 +2541,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
         <v>123</v>
       </c>
@@ -2525,13 +2558,13 @@
         <v>20</v>
       </c>
       <c r="F64" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="G64" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A65" t="s">
         <v>124</v>
       </c>
@@ -2539,7 +2572,7 @@
         <v>107</v>
       </c>
       <c r="C65" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="D65">
         <v>11</v>
@@ -2554,7 +2587,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A66" t="s">
         <v>125</v>
       </c>
@@ -2562,7 +2595,7 @@
         <v>8</v>
       </c>
       <c r="C66" t="s">
-        <v>84</v>
+        <v>253</v>
       </c>
       <c r="D66">
         <v>9</v>
@@ -2577,7 +2610,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
         <v>126</v>
       </c>
@@ -2600,7 +2633,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A68" t="s">
         <v>128</v>
       </c>
@@ -2623,7 +2656,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A69" t="s">
         <v>129</v>
       </c>
@@ -2634,19 +2667,19 @@
         <v>20</v>
       </c>
       <c r="D69">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E69">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F69" t="s">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="G69" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
         <v>130</v>
       </c>
@@ -2657,10 +2690,10 @@
         <v>131</v>
       </c>
       <c r="D70">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E70">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F70" t="s">
         <v>21</v>
@@ -2669,7 +2702,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
         <v>132</v>
       </c>
@@ -2680,19 +2713,19 @@
         <v>116</v>
       </c>
       <c r="D71">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E71">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F71" t="s">
-        <v>21</v>
+        <v>244</v>
       </c>
       <c r="G71" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
         <v>133</v>
       </c>
@@ -2703,10 +2736,10 @@
         <v>134</v>
       </c>
       <c r="D72">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E72">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F72" t="s">
         <v>21</v>
@@ -2715,7 +2748,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
         <v>135</v>
       </c>
@@ -2729,7 +2762,7 @@
         <v>10</v>
       </c>
       <c r="E73">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F73" t="s">
         <v>21</v>
@@ -2738,7 +2771,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
         <v>136</v>
       </c>
@@ -2746,10 +2779,10 @@
         <v>137</v>
       </c>
       <c r="D74">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E74">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F74" t="s">
         <v>21</v>
@@ -2758,7 +2791,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A75" t="s">
         <v>138</v>
       </c>
@@ -2769,10 +2802,10 @@
         <v>119</v>
       </c>
       <c r="D75">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E75">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F75" t="s">
         <v>21</v>
@@ -2781,7 +2814,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A76" t="s">
         <v>139</v>
       </c>
@@ -2792,10 +2825,10 @@
         <v>122</v>
       </c>
       <c r="D76">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E76">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F76" t="s">
         <v>21</v>
@@ -2804,7 +2837,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A77" t="s">
         <v>140</v>
       </c>
@@ -2815,19 +2848,19 @@
         <v>73</v>
       </c>
       <c r="D77">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E77">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F77" t="s">
-        <v>21</v>
+        <v>245</v>
       </c>
       <c r="G77" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A78" t="s">
         <v>141</v>
       </c>
@@ -2850,13 +2883,16 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A79" t="s">
         <v>143</v>
       </c>
       <c r="B79" t="s">
         <v>29</v>
       </c>
+      <c r="C79" s="1" t="s">
+        <v>246</v>
+      </c>
       <c r="D79">
         <v>12</v>
       </c>
@@ -2870,7 +2906,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A80" t="s">
         <v>144</v>
       </c>
@@ -2887,13 +2923,13 @@
         <v>20</v>
       </c>
       <c r="F80" t="s">
-        <v>18</v>
+        <v>247</v>
       </c>
       <c r="G80" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A81" t="s">
         <v>145</v>
       </c>
@@ -2916,7 +2952,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A82" t="s">
         <v>147</v>
       </c>
@@ -2939,7 +2975,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A83" t="s">
         <v>148</v>
       </c>
@@ -2947,7 +2983,7 @@
         <v>8</v>
       </c>
       <c r="C83" t="s">
-        <v>84</v>
+        <v>253</v>
       </c>
       <c r="D83">
         <v>11</v>
@@ -2962,7 +2998,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A84" t="s">
         <v>149</v>
       </c>
@@ -2979,13 +3015,13 @@
         <v>14</v>
       </c>
       <c r="F84" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="G84" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A85" t="s">
         <v>150</v>
       </c>
@@ -3008,7 +3044,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A86" t="s">
         <v>152</v>
       </c>
@@ -3031,7 +3067,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A87" t="s">
         <v>153</v>
       </c>
@@ -3048,13 +3084,13 @@
         <v>20</v>
       </c>
       <c r="F87" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="G87" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A88" t="s">
         <v>154</v>
       </c>
@@ -3062,19 +3098,19 @@
         <v>8</v>
       </c>
       <c r="D88">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E88">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F88" t="s">
-        <v>21</v>
+        <v>248</v>
       </c>
       <c r="G88" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A89" t="s">
         <v>155</v>
       </c>
@@ -3085,30 +3121,30 @@
         <v>156</v>
       </c>
       <c r="D89">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E89">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F89" t="s">
-        <v>21</v>
+        <v>238</v>
       </c>
       <c r="G89" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A90" t="s">
         <v>157</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="1" t="s">
         <v>158</v>
       </c>
       <c r="D90">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E90">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F90" t="s">
         <v>21</v>
@@ -3117,27 +3153,30 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A91" t="s">
         <v>159</v>
       </c>
       <c r="B91" t="s">
         <v>8</v>
       </c>
+      <c r="C91" s="1" t="s">
+        <v>249</v>
+      </c>
       <c r="D91">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E91">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F91" t="s">
-        <v>21</v>
+        <v>220</v>
       </c>
       <c r="G91" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A92" t="s">
         <v>160</v>
       </c>
@@ -3148,19 +3187,19 @@
         <v>119</v>
       </c>
       <c r="D92">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E92">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F92" t="s">
-        <v>21</v>
+        <v>250</v>
       </c>
       <c r="G92" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A93" t="s">
         <v>161</v>
       </c>
@@ -3171,19 +3210,19 @@
         <v>162</v>
       </c>
       <c r="D93">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E93">
         <v>20</v>
       </c>
       <c r="F93" t="s">
-        <v>21</v>
+        <v>247</v>
       </c>
       <c r="G93" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A94" t="s">
         <v>163</v>
       </c>
@@ -3194,10 +3233,10 @@
         <v>17</v>
       </c>
       <c r="D94">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E94">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F94" t="s">
         <v>21</v>
@@ -3206,7 +3245,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A95" t="s">
         <v>164</v>
       </c>
@@ -3217,19 +3256,19 @@
         <v>165</v>
       </c>
       <c r="D95">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E95">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F95" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G95" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A96" t="s">
         <v>166</v>
       </c>
@@ -3240,10 +3279,10 @@
         <v>167</v>
       </c>
       <c r="D96">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E96">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F96" t="s">
         <v>21</v>
@@ -3252,7 +3291,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A97" t="s">
         <v>168</v>
       </c>
@@ -3263,19 +3302,19 @@
         <v>169</v>
       </c>
       <c r="D97">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E97">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F97" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G97" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A98" t="s">
         <v>170</v>
       </c>
@@ -3283,10 +3322,10 @@
         <v>43</v>
       </c>
       <c r="D98">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E98">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F98" t="s">
         <v>21</v>
@@ -3295,7 +3334,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A99" t="s">
         <v>171</v>
       </c>
@@ -3303,70 +3342,70 @@
         <v>8</v>
       </c>
       <c r="C99" t="s">
+        <v>251</v>
+      </c>
+      <c r="D99">
+        <v>7</v>
+      </c>
+      <c r="E99">
+        <v>19</v>
+      </c>
+      <c r="F99" t="s">
+        <v>21</v>
+      </c>
+      <c r="G99" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A100" t="s">
         <v>172</v>
       </c>
-      <c r="D99">
+      <c r="B100" t="s">
+        <v>173</v>
+      </c>
+      <c r="C100" t="s">
+        <v>174</v>
+      </c>
+      <c r="D100">
+        <v>11</v>
+      </c>
+      <c r="E100">
+        <v>19</v>
+      </c>
+      <c r="F100" t="s">
         <v>10</v>
       </c>
-      <c r="E99">
-        <v>20</v>
-      </c>
-      <c r="F99" t="s">
-        <v>21</v>
-      </c>
-      <c r="G99" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
-        <v>173</v>
-      </c>
-      <c r="B100" t="s">
-        <v>174</v>
-      </c>
-      <c r="C100" t="s">
+      <c r="G100" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A101" t="s">
         <v>175</v>
       </c>
-      <c r="D100">
-        <v>11</v>
-      </c>
-      <c r="E100">
-        <v>21</v>
-      </c>
-      <c r="F100" t="s">
-        <v>21</v>
-      </c>
-      <c r="G100" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A101" t="s">
+      <c r="B101" t="s">
+        <v>8</v>
+      </c>
+      <c r="C101" t="s">
+        <v>252</v>
+      </c>
+      <c r="D101">
+        <v>9</v>
+      </c>
+      <c r="E101">
+        <v>19</v>
+      </c>
+      <c r="F101" t="s">
+        <v>18</v>
+      </c>
+      <c r="G101" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A102" t="s">
         <v>176</v>
-      </c>
-      <c r="B101" t="s">
-        <v>8</v>
-      </c>
-      <c r="C101" t="s">
-        <v>20</v>
-      </c>
-      <c r="D101">
-        <v>10</v>
-      </c>
-      <c r="E101">
-        <v>20</v>
-      </c>
-      <c r="F101" t="s">
-        <v>21</v>
-      </c>
-      <c r="G101" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A102" t="s">
-        <v>177</v>
       </c>
       <c r="B102" t="s">
         <v>8</v>
@@ -3375,64 +3414,64 @@
         <v>73</v>
       </c>
       <c r="D102">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E102">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F102" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G102" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A103" t="s">
+        <v>177</v>
+      </c>
+      <c r="B103" t="s">
         <v>178</v>
       </c>
-      <c r="B103" t="s">
+      <c r="D103">
+        <v>18</v>
+      </c>
+      <c r="E103">
+        <v>23</v>
+      </c>
+      <c r="F103" t="s">
+        <v>21</v>
+      </c>
+      <c r="G103" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A104" t="s">
         <v>179</v>
       </c>
-      <c r="D103">
-        <v>11</v>
-      </c>
-      <c r="E103">
-        <v>22</v>
-      </c>
-      <c r="F103" t="s">
-        <v>21</v>
-      </c>
-      <c r="G103" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A104" t="s">
-        <v>180</v>
-      </c>
       <c r="B104" t="s">
         <v>8</v>
       </c>
       <c r="C104" t="s">
-        <v>84</v>
+        <v>253</v>
       </c>
       <c r="D104">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E104">
         <v>20</v>
       </c>
       <c r="F104" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G104" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A105" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B105" t="s">
         <v>8</v>
@@ -3441,21 +3480,21 @@
         <v>116</v>
       </c>
       <c r="D105">
+        <v>8</v>
+      </c>
+      <c r="E105">
+        <v>21</v>
+      </c>
+      <c r="F105" t="s">
         <v>10</v>
       </c>
-      <c r="E105">
-        <v>20</v>
-      </c>
-      <c r="F105" t="s">
-        <v>21</v>
-      </c>
       <c r="G105" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A106" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B106" t="s">
         <v>107</v>
@@ -3467,24 +3506,24 @@
         <v>11</v>
       </c>
       <c r="E106">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F106" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G106" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A107" t="s">
+        <v>182</v>
+      </c>
+      <c r="B107" t="s">
+        <v>8</v>
+      </c>
+      <c r="C107" t="s">
         <v>183</v>
-      </c>
-      <c r="B107" t="s">
-        <v>8</v>
-      </c>
-      <c r="C107" t="s">
-        <v>184</v>
       </c>
       <c r="D107">
         <v>6</v>
@@ -3499,78 +3538,78 @@
         <v>15</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A108" t="s">
+        <v>184</v>
+      </c>
+      <c r="B108" t="s">
+        <v>8</v>
+      </c>
+      <c r="C108" t="s">
         <v>185</v>
       </c>
-      <c r="B108" t="s">
-        <v>8</v>
-      </c>
-      <c r="C108" t="s">
-        <v>186</v>
-      </c>
       <c r="D108">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E108">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F108" t="s">
-        <v>21</v>
+        <v>254</v>
       </c>
       <c r="G108" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A109" t="s">
+        <v>186</v>
+      </c>
+      <c r="B109" t="s">
+        <v>8</v>
+      </c>
+      <c r="C109" t="s">
         <v>187</v>
       </c>
-      <c r="B109" t="s">
-        <v>8</v>
-      </c>
-      <c r="C109" t="s">
+      <c r="D109">
+        <v>15</v>
+      </c>
+      <c r="E109">
+        <v>21</v>
+      </c>
+      <c r="F109" t="s">
+        <v>255</v>
+      </c>
+      <c r="G109" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A110" t="s">
         <v>188</v>
       </c>
-      <c r="D109">
-        <v>10</v>
-      </c>
-      <c r="E109">
-        <v>20</v>
-      </c>
-      <c r="F109" t="s">
-        <v>21</v>
-      </c>
-      <c r="G109" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A110" t="s">
+      <c r="B110" t="s">
+        <v>8</v>
+      </c>
+      <c r="C110" t="s">
         <v>189</v>
       </c>
-      <c r="B110" t="s">
-        <v>8</v>
-      </c>
-      <c r="C110" t="s">
+      <c r="D110">
+        <v>7</v>
+      </c>
+      <c r="E110">
+        <v>13</v>
+      </c>
+      <c r="F110" t="s">
+        <v>21</v>
+      </c>
+      <c r="G110" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A111" t="s">
         <v>190</v>
-      </c>
-      <c r="D110">
-        <v>10</v>
-      </c>
-      <c r="E110">
-        <v>20</v>
-      </c>
-      <c r="F110" t="s">
-        <v>21</v>
-      </c>
-      <c r="G110" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A111" t="s">
-        <v>192</v>
       </c>
       <c r="B111" t="s">
         <v>8</v>
@@ -3579,21 +3618,21 @@
         <v>17</v>
       </c>
       <c r="D111">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E111">
         <v>20</v>
       </c>
       <c r="F111" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G111" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A112" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B112" t="s">
         <v>43</v>
@@ -3611,9 +3650,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A113" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B113" t="s">
         <v>107</v>
@@ -3634,9 +3673,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A114" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B114" t="s">
         <v>8</v>
@@ -3645,56 +3684,56 @@
         <v>122</v>
       </c>
       <c r="D114">
+        <v>11</v>
+      </c>
+      <c r="E114">
+        <v>19</v>
+      </c>
+      <c r="F114" t="s">
         <v>10</v>
       </c>
-      <c r="E114">
-        <v>20</v>
-      </c>
-      <c r="F114" t="s">
-        <v>21</v>
-      </c>
       <c r="G114" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A115" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B115" t="s">
         <v>8</v>
       </c>
       <c r="C115" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D115">
         <v>10</v>
       </c>
       <c r="E115">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F115" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G115" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A116" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B116" t="s">
         <v>8</v>
       </c>
       <c r="C116" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D116">
         <v>10</v>
       </c>
       <c r="E116">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F116" t="s">
         <v>21</v>
@@ -3703,55 +3742,55 @@
         <v>11</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A117" t="s">
+        <v>197</v>
+      </c>
+      <c r="B117" t="s">
+        <v>8</v>
+      </c>
+      <c r="C117" t="s">
+        <v>185</v>
+      </c>
+      <c r="D117">
+        <v>12</v>
+      </c>
+      <c r="E117">
+        <v>21</v>
+      </c>
+      <c r="F117" t="s">
+        <v>250</v>
+      </c>
+      <c r="G117" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A118" t="s">
+        <v>198</v>
+      </c>
+      <c r="B118" t="s">
+        <v>8</v>
+      </c>
+      <c r="C118" t="s">
+        <v>185</v>
+      </c>
+      <c r="D118">
+        <v>6</v>
+      </c>
+      <c r="E118">
+        <v>15</v>
+      </c>
+      <c r="F118" t="s">
+        <v>80</v>
+      </c>
+      <c r="G118" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A119" t="s">
         <v>199</v>
-      </c>
-      <c r="B117" t="s">
-        <v>8</v>
-      </c>
-      <c r="C117" t="s">
-        <v>186</v>
-      </c>
-      <c r="D117">
-        <v>10</v>
-      </c>
-      <c r="E117">
-        <v>20</v>
-      </c>
-      <c r="F117" t="s">
-        <v>21</v>
-      </c>
-      <c r="G117" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A118" t="s">
-        <v>200</v>
-      </c>
-      <c r="B118" t="s">
-        <v>8</v>
-      </c>
-      <c r="C118" t="s">
-        <v>186</v>
-      </c>
-      <c r="D118">
-        <v>10</v>
-      </c>
-      <c r="E118">
-        <v>20</v>
-      </c>
-      <c r="F118" t="s">
-        <v>21</v>
-      </c>
-      <c r="G118" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A119" t="s">
-        <v>201</v>
       </c>
       <c r="B119" t="s">
         <v>8</v>
@@ -3760,44 +3799,44 @@
         <v>73</v>
       </c>
       <c r="D119">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E119">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F119" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G119" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A120" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B120" t="s">
         <v>58</v>
       </c>
       <c r="C120" t="s">
-        <v>175</v>
+        <v>256</v>
       </c>
       <c r="D120">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E120">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F120" t="s">
-        <v>21</v>
+        <v>238</v>
       </c>
       <c r="G120" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A121" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B121" t="s">
         <v>8</v>
@@ -3806,21 +3845,21 @@
         <v>73</v>
       </c>
       <c r="D121">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E121">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F121" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G121" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A122" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B122" t="s">
         <v>8</v>
@@ -3829,33 +3868,33 @@
         <v>169</v>
       </c>
       <c r="D122">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E122">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F122" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G122" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A123" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B123" t="s">
         <v>8</v>
       </c>
       <c r="C123" t="s">
-        <v>32</v>
+        <v>257</v>
       </c>
       <c r="D123">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E123">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F123" t="s">
         <v>21</v>
@@ -3864,32 +3903,32 @@
         <v>70</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A124" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B124" t="s">
         <v>8</v>
       </c>
       <c r="C124" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D124">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E124">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F124" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G124" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A125" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B125" t="s">
         <v>8</v>
@@ -3898,21 +3937,21 @@
         <v>73</v>
       </c>
       <c r="D125">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E125">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F125" t="s">
-        <v>21</v>
+        <v>247</v>
       </c>
       <c r="G125" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A126" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B126" t="s">
         <v>8</v>
@@ -3921,27 +3960,27 @@
         <v>169</v>
       </c>
       <c r="D126">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E126">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F126" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G126" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A127" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B127" t="s">
         <v>8</v>
       </c>
       <c r="C127" t="s">
-        <v>84</v>
+        <v>253</v>
       </c>
       <c r="D127">
         <v>10</v>
@@ -3950,21 +3989,21 @@
         <v>20</v>
       </c>
       <c r="F127" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="G127" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A128" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B128" t="s">
         <v>8</v>
       </c>
       <c r="C128" t="s">
-        <v>84</v>
+        <v>253</v>
       </c>
       <c r="D128">
         <v>10</v>
@@ -3973,15 +4012,15 @@
         <v>20</v>
       </c>
       <c r="F128" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="G128" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A129" t="s">
-        <v>211</v>
+        <v>258</v>
       </c>
       <c r="B129" t="s">
         <v>8</v>
@@ -3990,33 +4029,33 @@
         <v>20</v>
       </c>
       <c r="D129">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E129">
         <v>20</v>
       </c>
       <c r="F129" t="s">
-        <v>21</v>
+        <v>235</v>
       </c>
       <c r="G129" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A130" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B130" t="s">
         <v>8</v>
       </c>
       <c r="C130" t="s">
-        <v>84</v>
+        <v>253</v>
       </c>
       <c r="D130">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E130">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F130" t="s">
         <v>21</v>
@@ -4025,9 +4064,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A131" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B131" t="s">
         <v>8</v>
@@ -4036,10 +4075,10 @@
         <v>9</v>
       </c>
       <c r="D131">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E131">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F131" t="s">
         <v>21</v>
@@ -4048,15 +4087,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A132" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B132" t="s">
         <v>158</v>
       </c>
       <c r="D132">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E132">
         <v>22</v>
@@ -4068,32 +4107,32 @@
         <v>11</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A133" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B133" t="s">
+        <v>173</v>
+      </c>
+      <c r="C133" t="s">
         <v>174</v>
       </c>
-      <c r="C133" t="s">
-        <v>175</v>
-      </c>
       <c r="D133">
         <v>11</v>
       </c>
       <c r="E133">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F133" t="s">
         <v>21</v>
       </c>
       <c r="G133" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A134" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B134" t="s">
         <v>8</v>
@@ -4105,7 +4144,7 @@
         <v>10</v>
       </c>
       <c r="E134">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F134" t="s">
         <v>21</v>
@@ -4114,35 +4153,32 @@
         <v>11</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A135" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B135" t="s">
-        <v>8</v>
-      </c>
-      <c r="C135" t="s">
-        <v>218</v>
+        <v>158</v>
       </c>
       <c r="D135">
+        <v>11</v>
+      </c>
+      <c r="E135">
+        <v>21</v>
+      </c>
+      <c r="F135" t="s">
         <v>10</v>
       </c>
-      <c r="E135">
-        <v>20</v>
-      </c>
-      <c r="F135" t="s">
-        <v>21</v>
-      </c>
       <c r="G135" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A136" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B136" t="s">
-        <v>158</v>
+        <v>43</v>
       </c>
       <c r="D136">
         <v>11</v>
@@ -4151,18 +4187,18 @@
         <v>22</v>
       </c>
       <c r="F136" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G136" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A137" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B137" t="s">
-        <v>43</v>
+        <v>217</v>
       </c>
       <c r="D137">
         <v>11</v>
@@ -4177,210 +4213,213 @@
         <v>11</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A138" t="s">
+        <v>218</v>
+      </c>
+      <c r="B138" t="s">
+        <v>8</v>
+      </c>
+      <c r="C138" t="s">
+        <v>219</v>
+      </c>
+      <c r="D138">
+        <v>16</v>
+      </c>
+      <c r="E138">
+        <v>20</v>
+      </c>
+      <c r="F138" t="s">
+        <v>220</v>
+      </c>
+      <c r="G138" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A139" t="s">
         <v>221</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B139" t="s">
+        <v>43</v>
+      </c>
+      <c r="D139">
+        <v>11</v>
+      </c>
+      <c r="E139">
+        <v>22</v>
+      </c>
+      <c r="F139" t="s">
+        <v>21</v>
+      </c>
+      <c r="G139" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A140" t="s">
         <v>222</v>
       </c>
-      <c r="D138">
-        <v>11</v>
-      </c>
-      <c r="E138">
-        <v>21</v>
-      </c>
-      <c r="F138" t="s">
-        <v>21</v>
-      </c>
-      <c r="G138" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A139" t="s">
+      <c r="B140" t="s">
+        <v>8</v>
+      </c>
+      <c r="C140" t="s">
+        <v>165</v>
+      </c>
+      <c r="D140">
+        <v>5</v>
+      </c>
+      <c r="E140">
+        <v>12</v>
+      </c>
+      <c r="F140" t="s">
+        <v>14</v>
+      </c>
+      <c r="G140" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A141" t="s">
         <v>223</v>
       </c>
-      <c r="B139" t="s">
-        <v>8</v>
-      </c>
-      <c r="C139" t="s">
+      <c r="B141" t="s">
+        <v>8</v>
+      </c>
+      <c r="C141" t="s">
+        <v>32</v>
+      </c>
+      <c r="D141">
+        <v>7</v>
+      </c>
+      <c r="E141">
+        <v>15</v>
+      </c>
+      <c r="F141" t="s">
+        <v>21</v>
+      </c>
+      <c r="G141" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A142" t="s">
         <v>224</v>
       </c>
-      <c r="D139">
-        <v>4</v>
-      </c>
-      <c r="E139">
-        <v>20</v>
-      </c>
-      <c r="F139" t="s">
+      <c r="B142" t="s">
+        <v>8</v>
+      </c>
+      <c r="C142" t="s">
+        <v>119</v>
+      </c>
+      <c r="D142">
+        <v>11</v>
+      </c>
+      <c r="E142">
+        <v>21</v>
+      </c>
+      <c r="F142" t="s">
+        <v>18</v>
+      </c>
+      <c r="G142" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A143" t="s">
         <v>225</v>
       </c>
-      <c r="G139" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A140" t="s">
+      <c r="B143" t="s">
+        <v>8</v>
+      </c>
+      <c r="C143" t="s">
+        <v>259</v>
+      </c>
+      <c r="D143">
+        <v>11</v>
+      </c>
+      <c r="E143">
+        <v>21</v>
+      </c>
+      <c r="F143" t="s">
+        <v>18</v>
+      </c>
+      <c r="G143" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A144" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="B140" t="s">
-        <v>43</v>
-      </c>
-      <c r="D140">
-        <v>11</v>
-      </c>
-      <c r="E140">
-        <v>22</v>
-      </c>
-      <c r="F140" t="s">
-        <v>21</v>
-      </c>
-      <c r="G140" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A141" t="s">
+      <c r="B144" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C144" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="B141" t="s">
-        <v>8</v>
-      </c>
-      <c r="C141" t="s">
-        <v>165</v>
-      </c>
-      <c r="D141">
+      <c r="D144" s="1">
+        <v>6</v>
+      </c>
+      <c r="E144" s="1">
+        <v>14</v>
+      </c>
+      <c r="F144" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E141">
-        <v>20</v>
-      </c>
-      <c r="F141" t="s">
-        <v>21</v>
-      </c>
-      <c r="G141" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A142" t="s">
+      <c r="G144" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A145" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B142" t="s">
-        <v>8</v>
-      </c>
-      <c r="C142" t="s">
-        <v>32</v>
-      </c>
-      <c r="D142">
-        <v>7</v>
-      </c>
-      <c r="E142">
-        <v>15</v>
-      </c>
-      <c r="F142" t="s">
-        <v>21</v>
-      </c>
-      <c r="G142" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A143" t="s">
+      <c r="B145" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C145" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="B143" t="s">
-        <v>8</v>
-      </c>
-      <c r="C143" t="s">
-        <v>119</v>
-      </c>
-      <c r="D143">
-        <v>10</v>
-      </c>
-      <c r="E143">
-        <v>20</v>
-      </c>
-      <c r="F143" t="s">
-        <v>21</v>
-      </c>
-      <c r="G143" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A144" t="s">
-        <v>230</v>
-      </c>
-      <c r="B144" t="s">
-        <v>8</v>
-      </c>
-      <c r="C144" t="s">
-        <v>119</v>
-      </c>
-      <c r="D144">
-        <v>11</v>
-      </c>
-      <c r="E144">
-        <v>21</v>
-      </c>
-      <c r="F144" t="s">
-        <v>21</v>
-      </c>
-      <c r="G144" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A145" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="B145" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C145" s="1" t="s">
-        <v>232</v>
-      </c>
       <c r="D145" s="1">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E145" s="1">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F145" s="1" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="G145" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="146" spans="1:7" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A146" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="B146" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C146" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="D146" s="1">
-        <v>11</v>
-      </c>
-      <c r="E146" s="1">
-        <v>0</v>
-      </c>
-      <c r="F146" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G146" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A146" t="s">
+        <v>230</v>
+      </c>
+      <c r="B146" t="s">
+        <v>8</v>
+      </c>
+      <c r="C146" t="s">
+        <v>227</v>
+      </c>
+      <c r="D146">
+        <v>6</v>
+      </c>
+      <c r="E146">
+        <v>14</v>
+      </c>
+      <c r="F146" t="s">
+        <v>238</v>
+      </c>
+      <c r="G146" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A147" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B147" t="s">
         <v>8</v>
@@ -4389,130 +4428,107 @@
         <v>232</v>
       </c>
       <c r="D147">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E147">
+        <v>20</v>
+      </c>
+      <c r="F147" t="s">
         <v>14</v>
       </c>
-      <c r="F147" t="s">
-        <v>243</v>
-      </c>
       <c r="G147" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A148" t="s">
+        <v>233</v>
+      </c>
+      <c r="B148" t="s">
+        <v>8</v>
+      </c>
+      <c r="C148" t="s">
+        <v>234</v>
+      </c>
+      <c r="D148">
+        <v>8</v>
+      </c>
+      <c r="E148">
+        <v>17</v>
+      </c>
+      <c r="F148" t="s">
+        <v>235</v>
+      </c>
+      <c r="G148" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A149" t="s">
         <v>236</v>
       </c>
-      <c r="B148" t="s">
-        <v>8</v>
-      </c>
-      <c r="C148" t="s">
+      <c r="B149" t="s">
+        <v>8</v>
+      </c>
+      <c r="C149" t="s">
+        <v>240</v>
+      </c>
+      <c r="D149">
+        <v>7</v>
+      </c>
+      <c r="E149">
+        <v>14</v>
+      </c>
+      <c r="F149" t="s">
+        <v>235</v>
+      </c>
+      <c r="G149" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A150" t="s">
         <v>237</v>
       </c>
-      <c r="D148">
-        <v>8</v>
-      </c>
-      <c r="E148">
-        <v>20</v>
-      </c>
-      <c r="F148" t="s">
-        <v>14</v>
-      </c>
-      <c r="G148" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A149" t="s">
-        <v>238</v>
-      </c>
-      <c r="B149" t="s">
-        <v>8</v>
-      </c>
-      <c r="C149" t="s">
-        <v>239</v>
-      </c>
-      <c r="D149">
-        <v>8</v>
-      </c>
-      <c r="E149">
-        <v>17</v>
-      </c>
-      <c r="F149" t="s">
+      <c r="B150" t="s">
+        <v>8</v>
+      </c>
+      <c r="C150" t="s">
         <v>240</v>
       </c>
-      <c r="G149" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A150" t="s">
-        <v>241</v>
-      </c>
-      <c r="B150" t="s">
-        <v>8</v>
-      </c>
-      <c r="C150" t="s">
-        <v>245</v>
-      </c>
       <c r="D150">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E150">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F150" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="G150" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A151" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B151" t="s">
         <v>8</v>
       </c>
       <c r="C151" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="D151">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E151">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F151" t="s">
-        <v>240</v>
+        <v>18</v>
       </c>
       <c r="G151" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A152" t="s">
-        <v>244</v>
-      </c>
-      <c r="B152" t="s">
-        <v>8</v>
-      </c>
-      <c r="C152" t="s">
-        <v>245</v>
-      </c>
-      <c r="D152">
-        <v>11</v>
-      </c>
-      <c r="E152">
-        <v>21</v>
-      </c>
-      <c r="F152" t="s">
-        <v>18</v>
-      </c>
-      <c r="G152" t="s">
         <v>70</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Brothers Ramen spot
</commit_message>
<xml_diff>
--- a/food_spots.xlsx
+++ b/food_spots.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newsc\OneDrive\Documents\Cursor Projects\food-spot-selector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F36AB3C-3077-48A3-BF34-1A0C74A95629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9412421F-B8C3-49A3-AD76-04498C9F40DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10886" yWindow="0" windowWidth="11143" windowHeight="12429" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="12549" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="262">
   <si>
     <t>Place</t>
   </si>
@@ -800,6 +800,12 @@
   </si>
   <si>
     <t>Prawn Noodles, Hokkien Mee, Noodles</t>
+  </si>
+  <si>
+    <t>Brothers Ramen</t>
+  </si>
+  <si>
+    <t>Ramen, Noodles</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1129,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H151"/>
+  <dimension ref="A1:H152"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="16.921875" style="1" customWidth="1"/>
@@ -4532,6 +4538,29 @@
         <v>70</v>
       </c>
     </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A152" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="B152" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C152" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D152" s="1">
+        <v>11</v>
+      </c>
+      <c r="E152" s="1">
+        <v>19</v>
+      </c>
+      <c r="F152" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G152" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>